<commit_message>
Add project task list; update ranked retrieval docs, queries, and notebook
- Add documents/project_task_list.md tracking implementation phases
- Add detailed probabilistic IR / BM25 notes and update theory.md
- Refresh query generation notebook and queries_part_a.xlsx

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/evaluation/queries_part_a.xlsx
+++ b/data/evaluation/queries_part_a.xlsx
@@ -43,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,13 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2453,12 +2461,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>City Yatai Smart Industrial New</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>Yatai Smart Indsutrial New City</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Yatai Smart Industrial New Ciy</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2492,12 +2500,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
+          <t>Hrupp" Tovarystvo z obmezhenoiu vidpovidalnistiu "Zelinskyi</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
           <t>Tovarystvo z obmezhenoiu vidpvoidalnistiu "Zelinskyi Hrupp"</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Tovarystvo z obmezhenoiu vidpovidalnistiu "Zelinskyi Hrup"</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2531,12 +2539,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
+          <t>Nyrt. Ny. D. Zelinszkij EHMZ</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
           <t>Ny. D. Zelinszikj EHMZ Nyrt.</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Ny. D. Zelinszkij EHMZ Nyr.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2570,12 +2578,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
+          <t>"Mahistar-SH" Pryvatne pidpryiemstvo</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
           <t>Pryvatne pidpryiemtsvo "Mahistar-SH"</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Pryvatne pidpryiemstvo "Mahistar-S"</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2609,12 +2617,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
+          <t>"Elektroahrehat" Aktsionerne tovarystvo</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
           <t>Aktsionerne tovarysvto "Elektroahrehat"</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Aktsionerne tovarystvo "Elektroahreha"</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2648,12 +2656,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
+          <t>Leff Arnita Cowan</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
           <t>Arnita Cwoan Leff</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Arnita Cowan Lef</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2687,12 +2695,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
+          <t>Kuajian Michael</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>MichaelK uajian</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Michael Kuajin</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2726,12 +2734,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
+          <t>Hussain Yasin M.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
           <t>Yasin M.H ussain</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Yasin M. Hussan</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2765,12 +2773,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
+          <t>Ltd. Xinjiang Xinmuwei Clothing Co.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
           <t>Xinjiang Xinmuwei lCothing Co., Ltd.</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Xinjiang Xinmuwei Clothing Co., Lt.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2804,12 +2812,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
+          <t>Irakli Chanturiia</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
           <t>Chanturiai Irakli</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Chanturiia Iraki</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2843,12 +2851,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
+          <t>ПАРК OOO СПЕЦИАЛИЗИРОВАННЫЙ ЗАСТРОЙЩИК АЛАБУГА ЮЖНЫЙ</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t>OOO СПЕЦИАЛИЗИРОВАННЫЙ ЗАСРТОЙЩИК АЛАБУГА ЮЖНЫЙ ПАРК</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>OOO СПЕЦИАЛИЗИРОВАННЫЙ ЗАСТРОЙЩИК АЛАБУГА ЮЖНЫЙ ПАК</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2882,12 +2890,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
+          <t>AWARDS SD DIGITAL MARKETING</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
           <t>SD DIGITAL MAKRETING AWARDS</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>SD DIGITAL MARKETING AWARS</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2921,12 +2929,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
+          <t>kombinat» Tovarystvo z obmezhenoiu vidpovidalnistiu «Sychovskyi vyrobnycho-tekhnolohichnyi</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
           <t>Tovarystvo z obmezhenoiu vidpovidalnistiu «Syhcovskyi vyrobnycho-tekhnolohichnyi kombinat»</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Tovarystvo z obmezhenoiu vidpovidalnistiu «Sychovskyi vyrobnycho-tekhnolohichnyi kombina»</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2960,12 +2968,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
+          <t>Yuriiovych Starovoitov Stanislav</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
           <t>Starovoitov Stansilav Yuriiovych</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Starovoitov Stanislav Yuriiovyh</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2999,12 +3007,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
+          <t>"ЭКВИК" ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
           <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ТОВЕТСТВЕННОСТЬЮ "ЭКВИК"</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ЭКВИ"</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3038,12 +3046,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
+          <t>Викторович Маслов Алексей</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>Маслов Алексйе Викторович</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Маслов Алексей Викторовч</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3077,12 +3085,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
+          <t>Haas Renee M.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>Renee .M Haas</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Renee M. Has</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3116,12 +3124,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
+          <t>河北建设集团股份有限公司无极县分公司</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
           <t>河北建设集团股份有公限司无极县分公司</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>河北建设集团股份有限公司无极县分司</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3155,12 +3163,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
+          <t>Rosiia» Tovarystvo z obmezhenoiu vidpovidalnistiu «DZh.T.I.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
           <t>Tovarystvo z obmezhenoiu vidpvoidalnistiu «DZh.T.I. Rosiia»</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Tovarystvo z obmezhenoiu vidpovidalnistiu «DZh.T.I. Rosii»</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3194,12 +3202,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
+          <t>LLC Labsource</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
           <t>Labsourec, LLC</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Labsource, LC</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3233,12 +3241,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
+          <t>Serhiiovych Luzhbin Ihor</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
           <t>Luzhbin IhorS erhiiovych</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Luzhbin Ihor Serhiiovyh</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3272,12 +3280,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
+          <t>Rosiyi" Federalne kazenne pidpryiemstvo "Natsionalne vyprobuvalne obiednannia "Derzhavni boieprypasni vyprobuvalni polihony</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>Federalne kazenne pidpryiemstvo "Natsionalne vyprobuvalne obidenannia "Derzhavni boieprypasni vyprobuvalni polihony Rosiyi"</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Federalne kazenne pidpryiemstvo "Natsionalne vyprobuvalne obiednannia "Derzhavni boieprypasni vyprobuvalni polihony Rosiy"</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3311,12 +3319,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
+          <t>星龍興業有限公司</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
           <t>星龍興業限有公司</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>星龍興業有限司</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3350,12 +3358,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
+          <t>Chen Kan</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
           <t>Kan hCen</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>Kan Chn</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3389,12 +3397,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
+          <t>CORPORATION CITADEL ECONOMIC DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
           <t>CITADEL ECONOMIC DEVLEOPMENT CORPORATION</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>CITADEL ECONOMIC DEVELOPMENT CORPORATIN</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3428,12 +3436,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
+          <t>INC JUST 4 TODAY TRANSPORTATION</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
           <t>JUST 4 TODAY TRASNPORTATION, INC</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>JUST 4 TODAY TRANSPORTATION, IC</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3467,12 +3475,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
+          <t>Mykolayivna Baieva Kateryna</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
           <t>Baieva Kateryan Mykolayivna</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Baieva Kateryna Mykolayiva</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3506,12 +3514,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
+          <t>Mykolaiovych Holoborodko Pavlo</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
           <t>Holoborodko Pavol Mykolaiovych</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>Holoborodko Pavlo Mykolaiovyh</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3545,12 +3553,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
+          <t>赣州集达建筑工程有限公司</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
           <t>赣州集达建筑程工有限公司</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>赣州集达建筑工程有限司</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3584,12 +3592,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
+          <t>AYODEJI FASONU</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
           <t>FASONU,A YODEJI</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>FASONU, AYODEI</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3623,12 +3631,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
+          <t>EDEM EDEDEM EKPENYONG</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
           <t>EDEDEM EKPNEYONG EDEM</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>EDEDEM EKPENYONG EDM</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3662,12 +3670,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
+          <t>Avto" Tovarystvo z obmezhenoiu vidpovidalnistiu "MTS</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
           <t>Tovarystvo z obmezhenoiu vdipovidalnistiu "MTS Avto"</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Tovarystvo z obmezhenoiu vidpovidalnistiu "MTS Avt"</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3701,12 +3709,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
+          <t>ПРО' ООО 'ЭЛЕКТРА</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
           <t>ООО 'ЭЛЕТКРА ПРО'</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>ООО 'ЭЛЕКТРА ПР'</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3740,12 +3748,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
+          <t>Baatrovych Sanhadzhy-Horiaiev Dzhanhar</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
           <t>Sanhadzhy-Horiaiev zDhanhar Baatrovych</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Sanhadzhy-Horiaiev Dzhanhar Baatrovyh</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3779,12 +3787,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
+          <t>Volodymyrivna Korsakova Tetiana</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
           <t>Korsakova Tetiaan Volodymyrivna</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>Korsakova Tetiana Volodymyriva</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3818,12 +3826,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
+          <t>Mr. Dominguez Néstor Alfredo Domínguez Hernández</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
           <t>Néstor Alfredo DomínguezH ernández, Mr. Dominguez</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>Néstor Alfredo Domínguez Hernández, Mr. Dominguz</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3857,12 +3865,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
+          <t>Anatoliyivna Kostenko Iryna</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
           <t>Kostenko Iryn aAnatoliyivna</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Kostenko Iryna Anatoliyiva</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3896,12 +3904,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
+          <t>ANITA TREGO-CAMPION</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
           <t>TREGO-CAMPOIN, ANITA</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>TREGO-CAMPION, ANIA</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3935,12 +3943,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
+          <t>SIROIS JAMES R.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
           <t>JAMES R .SIROIS</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>JAMES R. SIROS</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3974,12 +3982,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
+          <t>Iraklii Rekhviashvili</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
           <t>Rekhviashvlii Iraklii</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Rekhviashvili Irakli</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4013,12 +4021,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
+          <t>Viktorivna Isaienko Viktoriia</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
           <t>Isaienko Viktoiria Viktorivna</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Isaienko Viktoriia Viktoriva</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4052,12 +4060,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
+          <t>Technology Scientific and Production Association of Measuring</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
           <t>Scientific and Production Assoication of Measuring Technology</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Scientific and Production Association of Measuring Technoloy</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4091,12 +4099,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
+          <t>JADALI Bahrami Ali</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
           <t>Bahrami Ail JADALI</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Bahrami Ali JADAI</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4130,12 +4138,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
+          <t>LLC Golden Luxury Jewellery Trading</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
           <t>Golden Luxury Jewlelery Trading LLC</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Golden Luxury Jewellery Trading LC</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4169,12 +4177,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
+          <t>Vasylovych Riakhovskyi Serhii</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
           <t>Riakhovskyi Sehrii Vasylovych</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Riakhovskyi Serhii Vasylovyh</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4208,12 +4216,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
+          <t>(JRA) Japanese Red Army</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
           <t>Japanese Re dArmy (JRA)</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Japanese Red Army (JR)</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4247,12 +4255,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
+          <t>AL-JAZA'IRI Usama Abu-'Abd-al-Wahid</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
           <t>Usama Abu-'Abd-alW-ahid AL-JAZA'IRI</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Usama Abu-'Abd-al-Wahid AL-JAZA'II</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4286,12 +4294,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
+          <t>Yuriyivna Veber Mariia</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
           <t>Veber Marii aYuriyivna</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Veber Mariia Yuriyiva</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4325,12 +4333,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
+          <t>Patricia Melia</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
           <t>Melia, aPtricia</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Melia, Patrica</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -4364,12 +4372,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
+          <t>ZKX SemiCore</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
           <t>SemiCoer ZKX</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>SemiCore ZX</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -4413,7 +4421,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>no-nbim-73bdf485c77b97920d6cb22d7cd2dbb8230862a5; no-nbim-bf2d032b20742e96ae44babaa466c3cdadd78663; no-nbim-1beff25f934cee1598161e40b471b52123df54c9; no-nbim-c78a34b47f6f3c85ead2bccd7c1e3e7503801a95; no-nbim-b90d5cd1d396053868a7b9e020d58f7754912ad5; no-nbim-dd5ab3dc28c26fcb513dff359d17ce515eea3183; no-nbim-63a600f743bfe956b9df2af24a7b32125648d180; no-nbim-bd2c52cc245ac8e55b0e575283682c74d3f87516; no-nbim-87924e102df77fa23c073a33bcd066d620a9f07f; no-nbim-1bab50d2c7a294a7323a6dcf2f497f709118abb9; no-nbim-6263fbd15decf3fa94e6144b5d081e041c0e986c; no-nbim-c2a31abfe03f36837644ad3332432c0f121e992d; no-nbim-0caa5c5762286eab920dfcce0e402d821197e406; no-nbim-e1a42a8ae233c9144f4d0ca36cc2ffbda8109965; no-nbim-6e58011b6fb22245db2ec396f115fa7b05f43a8d; no-nbim-621da685abf98b1e2255bbde8a3a214bf5fc7d25; no-nbim-796013e4261b5a4a88a6c5853ec7083785d96d7f; no-nbim-f3ca280a749f3cc4b0733ee9724f28f663f70322; no-nbim-fe57f3867628df5490b8de79359e8b9440f7b108; no-nbim-3d3dd0659fdbd1c75694a2da105a6e99ca2febf6; no-nbim-b82fc7b10e36cc391e0ccfa0afe55d219fede3fd; no-nbim-ddc88247fe7b3458f51144a5dfd07db27781aa37; no-nbim-804c2ea28eb68db241f29249a13827e8290d6ad3; no-nbim-ee71258415a706a211f380dc2cc8feb057f028a2; no-nbim-74f3598b9975a10d1f8ecc8859f5702f2a7ab84d; no-nbim-38f9e430e2eb92c832fb872620a363b83bf6f1be; no-nbim-7cea9eb3485e897f3718760d5ebd4a89717aea13; no-nbim-c2c14c0a811b0eed77d6f2d3e0dacf3c31b34122; no-nbim-b08d2577f248c8b1d39b08435dbbd0e9afa59fa8; no-nbim-9b85dab6c6175df3506bc0960955b0ba384469b6; no-nbim-c31d91f4b3e5c4b12a04b5fa7bf67b8f17f9881c; no-nbim-cafaac304fdba58e3473b57822848a7653887134; no-nbim-67c789be187a8f7a184e97c9b86c62747ea63a6f; no-nbim-8f2d54f562811096efc0f8fcd94da387d4065213; no-nbim-159d40231ae5455d48893546feb071a44ace7ad5; no-nbim-3da207f65df004979818399e2527af8488030177; no-nbim-2fb09d703cbae64bae53096f662168f8e6559fb0; no-nbim-2ee9948ed42f3eeb4e9ecfd4a64e715b8d92e4c2; no-nbim-9a5dde38aba3dc077cba72e92bc55a9048d9e065; no-nbim-330707a269a23eaa4ed0a1f704c24ac0bbfb503c; no-nbim-c42fff5759835bb3d9cb75e3d8ba077b996e4e6a; no-nbim-b2140bf41caf38f52b626624e29eded4bada394a; no-nbim-b4630a55772a9fc1cb03763261dae20a6558d7e3; no-nbim-a47fb56985532a7a7bce4d3eca88be7fa2a18ec4; no-nbim-d61e9a8b13306b88a4215e055ec034f3486719d7; no-nbim-95b9121e72ba3a5bf5841f46b8f1ac17e68d9a9f; no-nbim-de11858b95048a91dd053593b48ab67238cfe34d; no-nbim-1506cdc8b73168848c19cb8cf3444e6cfcadd742; no-nbim-ef7cd2460d64f11f4a0f76798a4357d9c1391b54; no-nbim-81b92a5bf60c13bc18d5e3057e0b6506082e0ecd; no-nbim-730e90a05b69ca08afe4b0000712ce8fb50c5552; no-nbim-6fff0d33812ca525821ac126b668c157cb2dadb3; no-nbim-d2c81029debad5d682d8f5c809f3b41c1b97ed85; no-nbim-9a30ee913632364d8454d44366d64b2260e27973; no-nbim-b5491e4ce61db8e2a06ef8efba2634a6f3b29472; no-nbim-d1d8f5584368072877a1e642ae39c598554b30e9; no-nbim-050c2b2b26073cafdaf765f52ae7172fc2480cc9; no-nbim-3b7a452e42023cd81364af5810d88a6191bdb7dd; no-nbim-5da646e195992ea00de285f439331c0313fd765e; no-nbim-1c325cae92a99ff434adeb885f254e6cdce2fb23; no-nbim-be943779c692b45c2c3cd3255151263f69a2479e; no-nbim-0efbf06b116806667c55652c6da9050471bda47f; no-nbim-fcb700a37c3d71193720c6e3ab0edef59ee64b3d; no-nbim-ade1c8f19caf6496bf7f28535570cd3e96c97894; no-nbim-f0342c9dc21d149138c14beb429b3d00306b312a; no-nbim-c86847f5dbe7dd574ff5f1d69d63f4bb116df62d; no-nbim-fb6018b447bbc40c3a5c32c51cecc1731940166c; no-nbim-82dde6bd6b9b4874adb6ab584b3c202acb5e5ae3; no-nbim-88fccaa43a9727ef731ebe0a68975cebde766a8e; no-nbim-e3d7a1d6b9e538503945fda52329836ef4c5e12a; no-nbim-6963aa70f8bc1065afa55044309c539e200e76fe; no-nbim-3a5ef37a435633c40917e8b687af37e372b3ebbe; no-nbim-65ecf76f6ac314cf50a43772e53b53f39b31faf2; no-nbim-eb10adc337c95028446d35769d0b6df3c1caf788; no-nbim-7cf8abeaa6a12c913eb35207ebefc504440be719; no-nbim-a0a964a7a911acc13fa5a3da83840bd2704ded49; no-nbim-e2eb51a6760d2825ccd2fa5567274fb95a10ea49; no-nbim-1e7f2a407934bd09858653996f98358104db95c6; no-nbim-431a88d91a93b175def555e40b34651101fde85c; no-nbim-78befac8721edc5e793fba267238907ba8213f0f; no-nbim-889194d9d394477fb4eb10ac19ad56122d55863f; no-nbim-5b72c3bc1fb4744407162a2c0bc07ce62ff5e662; no-nbim-90d90f9c85972361be5367497f2fd9d660e66958; no-nbim-b8bee78b0805cd0c5b1555f60284d7b73e9e496b; no-nbim-303cbb54a28d4f62fb1e7816842943069cc90842; no-nbim-2c4c36430e841be3249b50bfcd4854d75c0bd0e9; no-nbim-350f5d64493c6e6db84cc98cc2678fd69b9f3f40; no-nbim-51b762e0d8ce521b776099612039ebada5dd4977; no-nbim-5e3c08a84f6bf86f34f125c7ff0d15aca7571765; no-nbim-11dbe7cd30f588dbf142d6a8bf05e01c8dbfdc3d; no-nbim-d8ba644cdb60202fdefa29ec5b52977f9660d6ef; no-nbim-e868d59916cdce206dce8dd9a87e96447aba87e5; no-nbim-b5ffaebe157f355ce2317383256437b3f007e6b3; no-nbim-ca86b11d6a04fe6dff6519092f4c2d431a9ffaa6; no-nbim-7e192c6f47e3f9d20f6db580a2a0e68855ebbfc1; no-nbim-5e181bca7ed78f522d666a1e7bf3d9acfd61dfb0; no-nbim-66c31ef33d29e1b522c88ce223960c4caccabbce; no-nbim-a5f6f61ebfb565a60edf8057889e366f65341225; no-nbim-f90e0e562feba37217f6ca6e81dd3f0d7f76736b; no-nbim-ccc5b5ecb4e97e2c6e7ec458ab090a64fff700db; no-nbim-234b01471c8df5c244116df53bea7aa3cd6d6d3a; no-nbim-2fd2ea3833ec746e47c74cd4ee9e7d6a425ab7d1</t>
+          <t>no-nbim-d8ba644cdb60202fdefa29ec5b52977f9660d6ef; no-nbim-66c31ef33d29e1b522c88ce223960c4caccabbce; no-nbim-1beff25f934cee1598161e40b471b52123df54c9; no-nbim-ef7cd2460d64f11f4a0f76798a4357d9c1391b54; no-nbim-9a30ee913632364d8454d44366d64b2260e27973; no-nbim-63a600f743bfe956b9df2af24a7b32125648d180; no-nbim-67c789be187a8f7a184e97c9b86c62747ea63a6f; no-nbim-a0a964a7a911acc13fa5a3da83840bd2704ded49; no-nbim-87924e102df77fa23c073a33bcd066d620a9f07f; no-nbim-38f9e430e2eb92c832fb872620a363b83bf6f1be; no-nbim-ccc5b5ecb4e97e2c6e7ec458ab090a64fff700db; no-nbim-d1d8f5584368072877a1e642ae39c598554b30e9; no-nbim-e2eb51a6760d2825ccd2fa5567274fb95a10ea49; no-nbim-b8bee78b0805cd0c5b1555f60284d7b73e9e496b; no-nbim-82dde6bd6b9b4874adb6ab584b3c202acb5e5ae3; no-nbim-8f2d54f562811096efc0f8fcd94da387d4065213; no-nbim-fb6018b447bbc40c3a5c32c51cecc1731940166c; no-nbim-9b85dab6c6175df3506bc0960955b0ba384469b6; no-nbim-fe57f3867628df5490b8de79359e8b9440f7b108; no-nbim-78befac8721edc5e793fba267238907ba8213f0f; no-nbim-74f3598b9975a10d1f8ecc8859f5702f2a7ab84d; no-nbim-050c2b2b26073cafdaf765f52ae7172fc2480cc9; no-nbim-bd2c52cc245ac8e55b0e575283682c74d3f87516; no-nbim-3a5ef37a435633c40917e8b687af37e372b3ebbe; no-nbim-5da646e195992ea00de285f439331c0313fd765e; no-nbim-51b762e0d8ce521b776099612039ebada5dd4977; no-nbim-5b72c3bc1fb4744407162a2c0bc07ce62ff5e662; no-nbim-81b92a5bf60c13bc18d5e3057e0b6506082e0ecd; no-nbim-f0342c9dc21d149138c14beb429b3d00306b312a; no-nbim-730e90a05b69ca08afe4b0000712ce8fb50c5552; no-nbim-9a5dde38aba3dc077cba72e92bc55a9048d9e065; no-nbim-7cf8abeaa6a12c913eb35207ebefc504440be719; no-nbim-3d3dd0659fdbd1c75694a2da105a6e99ca2febf6; no-nbim-c31d91f4b3e5c4b12a04b5fa7bf67b8f17f9881c; no-nbim-431a88d91a93b175def555e40b34651101fde85c; no-nbim-c2a31abfe03f36837644ad3332432c0f121e992d; no-nbim-d2c81029debad5d682d8f5c809f3b41c1b97ed85; no-nbim-b5ffaebe157f355ce2317383256437b3f007e6b3; no-nbim-1e7f2a407934bd09858653996f98358104db95c6; no-nbim-b5491e4ce61db8e2a06ef8efba2634a6f3b29472; no-nbim-a47fb56985532a7a7bce4d3eca88be7fa2a18ec4; no-nbim-7e192c6f47e3f9d20f6db580a2a0e68855ebbfc1; no-nbim-2ee9948ed42f3eeb4e9ecfd4a64e715b8d92e4c2; no-nbim-3da207f65df004979818399e2527af8488030177; no-nbim-ddc88247fe7b3458f51144a5dfd07db27781aa37; no-nbim-f3ca280a749f3cc4b0733ee9724f28f663f70322; no-nbim-2fb09d703cbae64bae53096f662168f8e6559fb0; no-nbim-621da685abf98b1e2255bbde8a3a214bf5fc7d25; no-nbim-f90e0e562feba37217f6ca6e81dd3f0d7f76736b; no-nbim-fcb700a37c3d71193720c6e3ab0edef59ee64b3d; no-nbim-5e3c08a84f6bf86f34f125c7ff0d15aca7571765; no-nbim-d61e9a8b13306b88a4215e055ec034f3486719d7; no-nbim-1506cdc8b73168848c19cb8cf3444e6cfcadd742; no-nbim-3b7a452e42023cd81364af5810d88a6191bdb7dd; no-nbim-2fd2ea3833ec746e47c74cd4ee9e7d6a425ab7d1; no-nbim-e868d59916cdce206dce8dd9a87e96447aba87e5; no-nbim-5e181bca7ed78f522d666a1e7bf3d9acfd61dfb0; no-nbim-804c2ea28eb68db241f29249a13827e8290d6ad3; no-nbim-b4630a55772a9fc1cb03763261dae20a6558d7e3; no-nbim-234b01471c8df5c244116df53bea7aa3cd6d6d3a; no-nbim-0efbf06b116806667c55652c6da9050471bda47f; no-nbim-1c325cae92a99ff434adeb885f254e6cdce2fb23; no-nbim-e1a42a8ae233c9144f4d0ca36cc2ffbda8109965; no-nbim-6963aa70f8bc1065afa55044309c539e200e76fe; no-nbim-95b9121e72ba3a5bf5841f46b8f1ac17e68d9a9f; no-nbim-b08d2577f248c8b1d39b08435dbbd0e9afa59fa8; no-nbim-be943779c692b45c2c3cd3255151263f69a2479e; no-nbim-0caa5c5762286eab920dfcce0e402d821197e406; no-nbim-cafaac304fdba58e3473b57822848a7653887134; no-nbim-c86847f5dbe7dd574ff5f1d69d63f4bb116df62d; no-nbim-2c4c36430e841be3249b50bfcd4854d75c0bd0e9; no-nbim-b82fc7b10e36cc391e0ccfa0afe55d219fede3fd; no-nbim-a5f6f61ebfb565a60edf8057889e366f65341225; no-nbim-e3d7a1d6b9e538503945fda52329836ef4c5e12a; no-nbim-ee71258415a706a211f380dc2cc8feb057f028a2; no-nbim-c42fff5759835bb3d9cb75e3d8ba077b996e4e6a; no-nbim-159d40231ae5455d48893546feb071a44ace7ad5; no-nbim-eb10adc337c95028446d35769d0b6df3c1caf788; no-nbim-dd5ab3dc28c26fcb513dff359d17ce515eea3183; no-nbim-889194d9d394477fb4eb10ac19ad56122d55863f; no-nbim-6e58011b6fb22245db2ec396f115fa7b05f43a8d; no-nbim-bf2d032b20742e96ae44babaa466c3cdadd78663; no-nbim-de11858b95048a91dd053593b48ab67238cfe34d; no-nbim-ca86b11d6a04fe6dff6519092f4c2d431a9ffaa6; no-nbim-b90d5cd1d396053868a7b9e020d58f7754912ad5; no-nbim-7cea9eb3485e897f3718760d5ebd4a89717aea13; no-nbim-90d90f9c85972361be5367497f2fd9d660e66958; no-nbim-303cbb54a28d4f62fb1e7816842943069cc90842; no-nbim-1bab50d2c7a294a7323a6dcf2f497f709118abb9; no-nbim-350f5d64493c6e6db84cc98cc2678fd69b9f3f40; no-nbim-c78a34b47f6f3c85ead2bccd7c1e3e7503801a95; no-nbim-b2140bf41caf38f52b626624e29eded4bada394a; no-nbim-88fccaa43a9727ef731ebe0a68975cebde766a8e; no-nbim-796013e4261b5a4a88a6c5853ec7083785d96d7f; no-nbim-11dbe7cd30f588dbf142d6a8bf05e01c8dbfdc3d; no-nbim-6fff0d33812ca525821ac126b668c157cb2dadb3; no-nbim-65ecf76f6ac314cf50a43772e53b53f39b31faf2; no-nbim-ade1c8f19caf6496bf7f28535570cd3e96c97894; no-nbim-c2c14c0a811b0eed77d6f2d3e0dacf3c31b34122; no-nbim-6263fbd15decf3fa94e6144b5d081e041c0e986c; no-nbim-330707a269a23eaa4ed0a1f704c24ac0bbfb503c; no-nbim-73bdf485c77b97920d6cb22d7cd2dbb8230862a5</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
@@ -4452,7 +4460,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>no-nbim-8794bbf6d88310777801fdcebf08cf627feaf55f; no-nbim-b7a418f8029bd3ecf81c1501760576f58bf750dc; no-nbim-fdced820a94adfa9ea230fa71ddba574451f44e3; no-nbim-27b65ab6a993e4882242ae029883fe2cb2270bcb; no-nbim-2f22bf95fbd286459d21d3a36d86836cae210e7c; no-nbim-cbf26a242626ff71250698f606aa40a99ce98cdf; no-nbim-63a6606e136c735f43d2d0a89a39b6c0750b6b6f; no-nbim-7573bdef05f827a5d6f2f0b07fa8b01a3ca5157b; no-nbim-ab5fd345b710299175d213291641ce41bacb07eb; no-nbim-22dbccdd1ec9dc3906e03a969e8d627d7191131e; no-nbim-26ba35c37300f5b4b4ad08c1ae78ee3e30477407; no-nbim-8f9928ce8009512b01f2593992a242542df70a47; no-nbim-229885536d10bd94f471a501c864b09a1c387864; no-nbim-6afe49ebe81bac22f816c5af86f116383a190206; no-nbim-c2ed7f83fc5d3b1a4edeea7a9a8034822afb2a34; no-nbim-d5329925f044f7056c89a2423fb4574b23e6aaaa; no-nbim-e7bb771e88cb2b69307144abc41013dd096d3830; no-nbim-02b8f21a8eca3d22bb737832f9430b449d76cc33; no-nbim-1ef091b0443360ab5801a1004cce4f7da9088a4d; no-nbim-7e342695b81dae90e24dbaf344624adf3b1c7d8b; no-nbim-a6d2f9208bd63599fe6ee5f6ceb95d5cf78714c3; no-nbim-05ec714f89832f32ce8f548d2092b5f1f520416e; no-nbim-bdbaaa9d9608812b7ccb5d16dcd1d8f8fa5b6a35; no-nbim-6acbfa0b96d9fe0dd2bade51e867cf001ac9b9c5; no-nbim-6561452c9c7d18c5c9346826cafb296efa6ef870; no-nbim-12344a507f0d838885b3bf90021b8dc35ebce1ae; no-nbim-db72171e5901f891e2d41f3a2588d0e711e6c70c; no-nbim-dc83820109e9b5a60c4511dd826d584c9ad6921e; no-nbim-9117947ec52d822f4268d41f8fcace342204d196; no-nbim-4fe9c4a9be5f445f8b76202b54ba2b2dc97fdc2a; no-nbim-af7062a6f52602169c8e8fe3c31ed751801f1538; no-nbim-edaf568a7f4b312cdc989209ab49dd027119e943; no-nbim-2a102e5081bd08f02c886165624afd09b9402c91; no-nbim-ca708c792fa6ae116ee00248928f8a439fe82808; no-nbim-dddedccd90848bb5118def1417688f4198fdae49; no-nbim-b104ce18553fbe819c6b58f396e363a83d0a542b; no-nbim-bcfab2235a6ce045967d03878aa82e1ad6a6c75a; no-nbim-0100b85d41846a9ad64492d85e8d32f24f3a8cff; no-nbim-33eba4515ab82121e82a40ccc3466a4efb77af51; no-nbim-61ecf6cb9f765959641d84c2246eed03f56a8221; no-nbim-11266744ed30d8426eeccb0c682262e88166173d; no-nbim-6bc98ba17ebbbcbbc2a559b4287f21b60437e7de; no-nbim-005da79574c3c9e30892461a3dec7d8cbaae5f83; no-nbim-5677917a8644c486e109d0e27bb955f7e426605e; no-nbim-7dcdaf1558218b9dfcc1a94964d942345f340c21; no-nbim-6c4e0af83f6cbc36b450e638fb11509fd6da3f9e; no-nbim-2a0e7196bf1eb9f75141f7a7966c071ea4d9d04c; no-nbim-5a3555db431f6f83cff8ea12547b3dd09be10cef; no-nbim-4ab546495e328586ce62a448ddc9a7ecbf3144b2; no-nbim-c68b4f4c80add95f91cd2108c25b4bbc7a810472; no-nbim-278e05831dedf955a8a9e75c921791bcb45dd5d5; no-nbim-5eb049e9cc3f95a6a0042ae9cc667f4bf805eaa1; no-nbim-2611455c26159c7d3a6a7cb0c59199fff5d8ca7b; no-nbim-5b32993d1bda680d678a2134f7e0ebb6c266b44f; no-nbim-86ae0c9e8f44fae6fe61f44e3eb3ea30bb3163f8; no-nbim-1d57b64f6e2b1a6bf4dcfa41de4d20a5ddbcbb40; no-nbim-5466ea0bda729a14afd913c74d8e828088a40f1e; no-nbim-afdadf16b5956e6bac58b6e3834f3133fc696157; no-nbim-f87f7c03c8f12e8cc59f88f02e91804d37033f5d; no-nbim-e1bc2bb6c458435aff9f022f5857bf1f8db73330; no-nbim-6327fc13fb7c282ed37934f5e802617089895aad; no-nbim-8a31b742cc0efbcc969b48f6dd2484d78c1b2a6f; no-nbim-201f2e6430c0d3a6aa44312d2611b4afeb20ec77; no-nbim-bc6751a6b538c594ac2d487205b5f3741d1dde9f; no-nbim-f6a1951203dba6598dc41cda5bb5f662e10f9482; no-nbim-6a22a03a2f43a40e1648b882ad89b7a093753bb9; no-nbim-8f926fe8ee4463bff3415f1acfc632e814a32e99; no-nbim-a15bf394c3d6e77a21be77eabb282e16393ce2b8; no-nbim-5d8526722c0646a7d80ef9c30888141c1b4b253a; no-nbim-dc47e4fa68ee842ea8c4ed5e3c827a407708807c; no-nbim-959a358e862195219eccf494de61be926aad83cd; no-nbim-9ad7de15726f2ed086dbb294db3145b9b08f244e; no-nbim-b28446444957073c9fb900caf46c65b233ad65e7; no-nbim-e8c1d2d2ba57c18e384a2b74ea798879ac355156</t>
+          <t>no-nbim-27b65ab6a993e4882242ae029883fe2cb2270bcb; no-nbim-bcfab2235a6ce045967d03878aa82e1ad6a6c75a; no-nbim-201f2e6430c0d3a6aa44312d2611b4afeb20ec77; no-nbim-a6d2f9208bd63599fe6ee5f6ceb95d5cf78714c3; no-nbim-6acbfa0b96d9fe0dd2bade51e867cf001ac9b9c5; no-nbim-6afe49ebe81bac22f816c5af86f116383a190206; no-nbim-e7bb771e88cb2b69307144abc41013dd096d3830; no-nbim-e1bc2bb6c458435aff9f022f5857bf1f8db73330; no-nbim-dc47e4fa68ee842ea8c4ed5e3c827a407708807c; no-nbim-12344a507f0d838885b3bf90021b8dc35ebce1ae; no-nbim-afdadf16b5956e6bac58b6e3834f3133fc696157; no-nbim-0100b85d41846a9ad64492d85e8d32f24f3a8cff; no-nbim-02b8f21a8eca3d22bb737832f9430b449d76cc33; no-nbim-c2ed7f83fc5d3b1a4edeea7a9a8034822afb2a34; no-nbim-61ecf6cb9f765959641d84c2246eed03f56a8221; no-nbim-cbf26a242626ff71250698f606aa40a99ce98cdf; no-nbim-5a3555db431f6f83cff8ea12547b3dd09be10cef; no-nbim-05ec714f89832f32ce8f548d2092b5f1f520416e; no-nbim-6561452c9c7d18c5c9346826cafb296efa6ef870; no-nbim-1d57b64f6e2b1a6bf4dcfa41de4d20a5ddbcbb40; no-nbim-1ef091b0443360ab5801a1004cce4f7da9088a4d; no-nbim-63a6606e136c735f43d2d0a89a39b6c0750b6b6f; no-nbim-959a358e862195219eccf494de61be926aad83cd; no-nbim-8f9928ce8009512b01f2593992a242542df70a47; no-nbim-a15bf394c3d6e77a21be77eabb282e16393ce2b8; no-nbim-6a22a03a2f43a40e1648b882ad89b7a093753bb9; no-nbim-8a31b742cc0efbcc969b48f6dd2484d78c1b2a6f; no-nbim-db72171e5901f891e2d41f3a2588d0e711e6c70c; no-nbim-e8c1d2d2ba57c18e384a2b74ea798879ac355156; no-nbim-ca708c792fa6ae116ee00248928f8a439fe82808; no-nbim-d5329925f044f7056c89a2423fb4574b23e6aaaa; no-nbim-b28446444957073c9fb900caf46c65b233ad65e7; no-nbim-6327fc13fb7c282ed37934f5e802617089895aad; no-nbim-7dcdaf1558218b9dfcc1a94964d942345f340c21; no-nbim-9117947ec52d822f4268d41f8fcace342204d196; no-nbim-af7062a6f52602169c8e8fe3c31ed751801f1538; no-nbim-b104ce18553fbe819c6b58f396e363a83d0a542b; no-nbim-2a0e7196bf1eb9f75141f7a7966c071ea4d9d04c; no-nbim-2f22bf95fbd286459d21d3a36d86836cae210e7c; no-nbim-6c4e0af83f6cbc36b450e638fb11509fd6da3f9e; no-nbim-c68b4f4c80add95f91cd2108c25b4bbc7a810472; no-nbim-dddedccd90848bb5118def1417688f4198fdae49; no-nbim-5b32993d1bda680d678a2134f7e0ebb6c266b44f; no-nbim-22dbccdd1ec9dc3906e03a969e8d627d7191131e; no-nbim-7573bdef05f827a5d6f2f0b07fa8b01a3ca5157b; no-nbim-bc6751a6b538c594ac2d487205b5f3741d1dde9f; no-nbim-86ae0c9e8f44fae6fe61f44e3eb3ea30bb3163f8; no-nbim-8794bbf6d88310777801fdcebf08cf627feaf55f; no-nbim-005da79574c3c9e30892461a3dec7d8cbaae5f83; no-nbim-f87f7c03c8f12e8cc59f88f02e91804d37033f5d; no-nbim-4ab546495e328586ce62a448ddc9a7ecbf3144b2; no-nbim-2a102e5081bd08f02c886165624afd09b9402c91; no-nbim-11266744ed30d8426eeccb0c682262e88166173d; no-nbim-b7a418f8029bd3ecf81c1501760576f58bf750dc; no-nbim-33eba4515ab82121e82a40ccc3466a4efb77af51; no-nbim-5466ea0bda729a14afd913c74d8e828088a40f1e; no-nbim-edaf568a7f4b312cdc989209ab49dd027119e943; no-nbim-278e05831dedf955a8a9e75c921791bcb45dd5d5; no-nbim-fdced820a94adfa9ea230fa71ddba574451f44e3; no-nbim-8f926fe8ee4463bff3415f1acfc632e814a32e99; no-nbim-f6a1951203dba6598dc41cda5bb5f662e10f9482; no-nbim-229885536d10bd94f471a501c864b09a1c387864; no-nbim-4fe9c4a9be5f445f8b76202b54ba2b2dc97fdc2a; no-nbim-5677917a8644c486e109d0e27bb955f7e426605e; no-nbim-5eb049e9cc3f95a6a0042ae9cc667f4bf805eaa1; no-nbim-7e342695b81dae90e24dbaf344624adf3b1c7d8b; no-nbim-9ad7de15726f2ed086dbb294db3145b9b08f244e; no-nbim-26ba35c37300f5b4b4ad08c1ae78ee3e30477407; no-nbim-5d8526722c0646a7d80ef9c30888141c1b4b253a; no-nbim-bdbaaa9d9608812b7ccb5d16dcd1d8f8fa5b6a35; no-nbim-dc83820109e9b5a60c4511dd826d584c9ad6921e; no-nbim-ab5fd345b710299175d213291641ce41bacb07eb; no-nbim-6bc98ba17ebbbcbbc2a559b4287f21b60437e7de; no-nbim-2611455c26159c7d3a6a7cb0c59199fff5d8ca7b</t>
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
@@ -4491,7 +4499,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>no-nbim-5c635e68e383978a47ab7bafc22f9d28c9288a33; no-nbim-cd90b207e7291cb38fed76363f72f3556f428eab; no-nbim-5410e3ac47aa4d50ebede788626f6595c33f8ffd; no-nbim-ab3776e7d93299c3295f0d5735d51e06bc90dde9; no-nbim-fed4d6f48b3a7ed22b9afdfe44c6fcd96e2335cf; no-nbim-bab628839d6060282fc141bc1e990ce88b271963; no-nbim-77c618dff09b05529a99bc6c1595b57acf04a9f0; no-nbim-087ed013485a52328e21953c5bcaa2ae959273c0; no-nbim-9b67daaa68170e4e0d062611524388c4f50cf6d0; no-nbim-df88e10477c03b4cfc530cd0e5d1744f82234f92; no-nbim-98bd75aa562faffe23b6be94fc87504784694d22; no-nbim-96074cfb2a61b57dc458cc61a58386298d15d1d0; no-nbim-bf30a020d61c2c128d70affdefb94af85de958a0; no-nbim-c940df0fca65dba9934ed92d9c8aa1f8b1bca193; no-nbim-3a79509473eca26d9708e932f94d9a9facb719df; no-nbim-771479d29387d24b0df80d2d14a179c646c9fb43; no-nbim-c120318bd4b2320ca4f6b0463d2635ccad90ae67; no-nbim-f430c99747a03fe42d8e3c9cf9f131d671d05bae; no-nbim-dcc8a5e2c8a67d410fc4660fc091acb6008f598d; no-nbim-7177a26dfb92b9423d89a02700fc8057f75c51af; no-nbim-5c00bbac742e672d7b6eea6632f7a03816ab74fe; no-nbim-945abfe111863feea13471b155985d641863f818; no-nbim-6aca56503d808b84a26703e5e1812865bf42e3eb; no-nbim-47b380051fe0efa2c3dc813113143ac6e9f7f7c7; no-nbim-7337ebc7f226ba0b9e979428efe238a6c76700be; no-nbim-7eff739c096a334de7917fad1cd343f10c75efd1; no-nbim-319173469c0162f082412a5ee9daf033f0f66fd3; no-nbim-933bf1a048f19afff587b8f3fe9375dfcaa551d5; no-nbim-9ab064602a9bd3434161d01f82b8af8a10c1784d; no-nbim-a39e3e17efae78653ebc6f18f43cf5876bd579c8; no-nbim-f266e2378558850a79abae180517098fac7b1c0e; no-nbim-b10102e2dbee0dbdf17c806640011ab6f1f7e55b; no-nbim-f146d0a97cedd17ce886ec021f05710ff624407e; no-nbim-8daf88ae08516af38cad1dfb31d681261815ae1c; no-nbim-23f5ad6b20e9292a6dcfa879798ecf8e6353d517; no-nbim-e91d18e17726149eb306dd0ec76f33c82c67cca2; no-nbim-a58711efd2e9dea7e2828408a314796aeef2371a; no-nbim-dd7a550bb001daa16bf3c3a00c69722cd5ae1841; no-nbim-27e266679e472b7398a521ae7e90bd4eb2d89fae; no-nbim-bdf8462befc085eb6a000c498853fc807d8a7fa6; no-nbim-06fe93e36164bc439b94d80a5f65e9202f8c770d; no-nbim-730ac4d166d52502f50e5f7b557309ed835d7f10; no-nbim-b01eb188d5980e0372b747ddf4382c1af0e37942; no-nbim-4c74ae7e058db34a0f66a81a1bae1d0a4672bd85; no-nbim-b61ac814d2d98675b854754244e9df81b71810f3; no-nbim-9c5f1a218b8c699151371a0c7c6a4557e870d290; no-nbim-aa365c737fc1726ae8dbbf47b6bff57df9f9da77; no-nbim-c8004d3f978a5e357ccac81c9718769b46381c22; no-nbim-8f7ce6ac619b41f6d3bb3d6a45f3aec733d0b2e5; no-nbim-ccf8ab4a7acf6db52fec0bf624890d8ffc62ddab; no-nbim-257d3452879fcb9a6834a271e4ba0b56716d2b20; no-nbim-15c6cdb4f7be9c7dca8c8fdccbeedbda07e5a3b1; no-nbim-2d5ce458433b87cb6ee4ee986ce56e403b92a5f7; no-nbim-fa345d47b282601d0193aeb0e0f79cef2063ed19; no-nbim-9179cb29a74c77457b7926509f71570700241abd; no-nbim-bc6600ca61a365cbee47ef9c54f4cdaf928afc5a; no-nbim-90fcd7a368f12aa95b37d89f615ee6d6c09175c9; no-nbim-d7c017411abbacca166746f6b102e84c68fb9d5a; no-nbim-a6d16dfc5337dcb8d2066164664c1e96a216f3e8; no-nbim-389934f3b21de026dcf500e1105370a12bca57c4; no-nbim-7e86f32a4198c21d5152dcf84fcee3a981d3cc5b; no-nbim-32ea4078520b350f463ef4ed4e87149ada8b0eb3; no-nbim-56e6ae14c2d556435e5939244a4b35dee3de2198; no-nbim-17f03d2aae44b125d58101632805b1ba7684f08b; no-nbim-650ab486d26454a1c2adb3d6d75e0114c32985a0; no-nbim-cc28e7b3d9f55d5a64787dff19abbc8cbea4d1cc; no-nbim-16e07ac7e88636eb443afec1d374bfccbdad5bb6; no-nbim-e1cb830e318ec203d12a08733c214e96aa8cc8d2; no-nbim-8f00c04b7f6a7a1c797b3987ccbc96081c829687</t>
+          <t>no-nbim-5c635e68e383978a47ab7bafc22f9d28c9288a33; no-nbim-4c74ae7e058db34a0f66a81a1bae1d0a4672bd85; no-nbim-6aca56503d808b84a26703e5e1812865bf42e3eb; no-nbim-98bd75aa562faffe23b6be94fc87504784694d22; no-nbim-16e07ac7e88636eb443afec1d374bfccbdad5bb6; no-nbim-7eff739c096a334de7917fad1cd343f10c75efd1; no-nbim-b01eb188d5980e0372b747ddf4382c1af0e37942; no-nbim-a58711efd2e9dea7e2828408a314796aeef2371a; no-nbim-a6d16dfc5337dcb8d2066164664c1e96a216f3e8; no-nbim-9ab064602a9bd3434161d01f82b8af8a10c1784d; no-nbim-771479d29387d24b0df80d2d14a179c646c9fb43; no-nbim-77c618dff09b05529a99bc6c1595b57acf04a9f0; no-nbim-9179cb29a74c77457b7926509f71570700241abd; no-nbim-cd90b207e7291cb38fed76363f72f3556f428eab; no-nbim-7177a26dfb92b9423d89a02700fc8057f75c51af; no-nbim-96074cfb2a61b57dc458cc61a58386298d15d1d0; no-nbim-27e266679e472b7398a521ae7e90bd4eb2d89fae; no-nbim-5c00bbac742e672d7b6eea6632f7a03816ab74fe; no-nbim-bab628839d6060282fc141bc1e990ce88b271963; no-nbim-945abfe111863feea13471b155985d641863f818; no-nbim-c940df0fca65dba9934ed92d9c8aa1f8b1bca193; no-nbim-e1cb830e318ec203d12a08733c214e96aa8cc8d2; no-nbim-389934f3b21de026dcf500e1105370a12bca57c4; no-nbim-650ab486d26454a1c2adb3d6d75e0114c32985a0; no-nbim-ccf8ab4a7acf6db52fec0bf624890d8ffc62ddab; no-nbim-47b380051fe0efa2c3dc813113143ac6e9f7f7c7; no-nbim-b10102e2dbee0dbdf17c806640011ab6f1f7e55b; no-nbim-257d3452879fcb9a6834a271e4ba0b56716d2b20; no-nbim-5410e3ac47aa4d50ebede788626f6595c33f8ffd; no-nbim-f266e2378558850a79abae180517098fac7b1c0e; no-nbim-df88e10477c03b4cfc530cd0e5d1744f82234f92; no-nbim-730ac4d166d52502f50e5f7b557309ed835d7f10; no-nbim-a39e3e17efae78653ebc6f18f43cf5876bd579c8; no-nbim-bf30a020d61c2c128d70affdefb94af85de958a0; no-nbim-17f03d2aae44b125d58101632805b1ba7684f08b; no-nbim-dcc8a5e2c8a67d410fc4660fc091acb6008f598d; no-nbim-e91d18e17726149eb306dd0ec76f33c82c67cca2; no-nbim-bc6600ca61a365cbee47ef9c54f4cdaf928afc5a; no-nbim-90fcd7a368f12aa95b37d89f615ee6d6c09175c9; no-nbim-8f7ce6ac619b41f6d3bb3d6a45f3aec733d0b2e5; no-nbim-cc28e7b3d9f55d5a64787dff19abbc8cbea4d1cc; no-nbim-fa345d47b282601d0193aeb0e0f79cef2063ed19; no-nbim-c120318bd4b2320ca4f6b0463d2635ccad90ae67; no-nbim-b61ac814d2d98675b854754244e9df81b71810f3; no-nbim-3a79509473eca26d9708e932f94d9a9facb719df; no-nbim-9c5f1a218b8c699151371a0c7c6a4557e870d290; no-nbim-7337ebc7f226ba0b9e979428efe238a6c76700be; no-nbim-8daf88ae08516af38cad1dfb31d681261815ae1c; no-nbim-f430c99747a03fe42d8e3c9cf9f131d671d05bae; no-nbim-7e86f32a4198c21d5152dcf84fcee3a981d3cc5b; no-nbim-8f00c04b7f6a7a1c797b3987ccbc96081c829687; no-nbim-23f5ad6b20e9292a6dcfa879798ecf8e6353d517; no-nbim-9b67daaa68170e4e0d062611524388c4f50cf6d0; no-nbim-f146d0a97cedd17ce886ec021f05710ff624407e; no-nbim-32ea4078520b350f463ef4ed4e87149ada8b0eb3; no-nbim-2d5ce458433b87cb6ee4ee986ce56e403b92a5f7; no-nbim-ab3776e7d93299c3295f0d5735d51e06bc90dde9; no-nbim-dd7a550bb001daa16bf3c3a00c69722cd5ae1841; no-nbim-319173469c0162f082412a5ee9daf033f0f66fd3; no-nbim-56e6ae14c2d556435e5939244a4b35dee3de2198; no-nbim-c8004d3f978a5e357ccac81c9718769b46381c22; no-nbim-bdf8462befc085eb6a000c498853fc807d8a7fa6; no-nbim-06fe93e36164bc439b94d80a5f65e9202f8c770d; no-nbim-d7c017411abbacca166746f6b102e84c68fb9d5a; no-nbim-aa365c737fc1726ae8dbbf47b6bff57df9f9da77; no-nbim-933bf1a048f19afff587b8f3fe9375dfcaa551d5; no-nbim-087ed013485a52328e21953c5bcaa2ae959273c0; no-nbim-fed4d6f48b3a7ed22b9afdfe44c6fcd96e2335cf; no-nbim-15c6cdb4f7be9c7dca8c8fdccbeedbda07e5a3b1</t>
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
@@ -4530,7 +4538,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>isin-RU000A10DDG3; isin-RU000A109783; isin-RU000A108CE5; isin-RU000A10BR02; isin-RU000A10DRV2; isin-RU000A109UL0; isin-RU000A10ARR6; isin-RU000A10CLZ8; isin-RU000A10AA77; isin-RU000A10BP46; isin-RU000A10D3R8; isin-RU000A10AYU6; isin-RU000A10AHP1; isin-RU000A108WJ2; isin-RU000A10DY35; isin-RU000A1082M3; isin-RU000A10DWP4; isin-RU000A10DYZ9; isin-RU000A10DEM9; isin-RU000A108LL1; isin-RU000A109KG1; isin-RU000A10A794; isin-RU000A10ASF9; isin-RU000A1097X8; isin-RU000A1084N7; isin-RU000A108FG3; isin-RU000A10BLP1; isin-RU000A10CM89; isin-RU000A109RX1; isin-RU000A10C873; isin-RU000A10CT09; isin-RU000A10DRX8; isin-RU000A10CSR0; isin-RU000A10EAQ6; isin-RU000A1098U2; isin-RU000A109AU3; isin-RU000A109MH5; isin-RU000A108UJ6; isin-RU000A109NM3; isin-RU000A10CRA8; isin-RU000A10DTB0; isin-RU000A108405; isin-RU000A10CM71; isin-RU000A10DBH5; isin-RU000A10BV89; isin-RU000A10CR92; isin-RU000A10D4E4; isin-RU000A1085A1; isin-RU000A109JX8; isin-RU000A10B2U6; isin-RU000A10E4F0; isin-RU000A10E7D8; isin-RU000A10AMP1; isin-RU000A107PM2; isin-RU000A108B83; isin-RU000A10A0H8; isin-RU000A10BGE5; isin-RU000A10A7A8; isin-RU000A1092T7; isin-RU000A10ED70; isin-RU000A109KK3; isin-RU000A10CM14; isin-RU000A10CAQ0</t>
+          <t>isin-RU000A108LL1; isin-RU000A108B83; isin-RU000A10BGE5; isin-RU000A10EAQ6; isin-RU000A10A0H8; isin-RU000A10ED70; isin-RU000A10ARR6; isin-RU000A109RX1; isin-RU000A108WJ2; isin-RU000A109KK3; isin-RU000A10C873; isin-RU000A10AMP1; isin-RU000A10CM89; isin-RU000A108FG3; isin-RU000A10CT09; isin-RU000A10BP46; isin-RU000A10DDG3; isin-RU000A10DTB0; isin-RU000A10CM71; isin-RU000A10CR92; isin-RU000A10CAQ0; isin-RU000A10DRX8; isin-RU000A1098U2; isin-RU000A10BLP1; isin-RU000A10E4F0; isin-RU000A10D4E4; isin-RU000A10CM14; isin-RU000A10DYZ9; isin-RU000A10BR02; isin-RU000A109UL0; isin-RU000A1084N7; isin-RU000A10AA77; isin-RU000A10AHP1; isin-RU000A10DBH5; isin-RU000A1085A1; isin-RU000A109AU3; isin-RU000A107PM2; isin-RU000A1092T7; isin-RU000A109KG1; isin-RU000A10DWP4; isin-RU000A10CRA8; isin-RU000A10DEM9; isin-RU000A10DY35; isin-RU000A108CE5; isin-RU000A108UJ6; isin-RU000A10A7A8; isin-RU000A10ASF9; isin-RU000A109783; isin-RU000A10AYU6; isin-RU000A10E7D8; isin-RU000A109NM3; isin-RU000A10BV89; isin-RU000A10DRV2; isin-RU000A108405; isin-RU000A1097X8; isin-RU000A10CSR0; isin-RU000A10B2U6; isin-RU000A10D3R8; isin-RU000A109JX8; isin-RU000A10CLZ8; isin-RU000A109MH5; isin-RU000A10A794; isin-RU000A1082M3</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -4569,7 +4577,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>isin-RU000A104A39; isin-RU000A106T85; isin-RU000A106DK4; isin-RU000A1021G3; isin-RU000A103935; isin-RU000A106938; isin-RU000A102RU2; isin-RU000A105YQ9; isin-RU000A105BP9; isin-RU000A101RF5; isin-RU000A106EV9; isin-RU000A105YA3; isin-RU000A106Y70; isin-RU000A1028C7; isin-RU000A1052T1; isin-RU000A103TV4; isin-RU000A105UZ8; isin-RU000A1064X8; isin-RU000A102B30; isin-RU000A107EC7; isin-RU000A105TR7; isin-RU000A102028; isin-RU000A1029A9; isin-RU000A103NJ2; isin-RU000A103RT2; isin-RU000A103W26; isin-RU000A103YP6; isin-RU000A1057A0; isin-RU000A1050X7; isin-RU000A104XW2; isin-RU000A107761; isin-RU000A105GS2; isin-RU000A103YF7; isin-RU000A102TT0; isin-RU000A103455; isin-RU000A107EW5; isin-RU000A1035D0; isin-RU000A105CS1; isin-RU000A105PR5; isin-RU000A1075D6; isin-RU000A103H25; isin-RU000A105SZ2; isin-RU000A1074F4; isin-RU000A105FM7; isin-RU000A105CL6; isin-RU000A1032S5; isin-RU000A104WS2; isin-RU000A104CJ3; isin-RU000A105Y14; isin-RU000A1034T9; isin-RU000A103WB0; isin-RU000A102LW1</t>
+          <t>isin-RU000A1050X7; isin-RU000A103935; isin-RU000A106938; isin-RU000A1028C7; isin-RU000A106EV9; isin-RU000A106DK4; isin-RU000A1052T1; isin-RU000A102TT0; isin-RU000A1075D6; isin-RU000A105PR5; isin-RU000A103YP6; isin-RU000A105TR7; isin-RU000A103W26; isin-RU000A104WS2; isin-RU000A103455; isin-RU000A103NJ2; isin-RU000A105BP9; isin-RU000A1029A9; isin-RU000A102028; isin-RU000A102RU2; isin-RU000A104XW2; isin-RU000A106Y70; isin-RU000A105CL6; isin-RU000A105YQ9; isin-RU000A103WB0; isin-RU000A105UZ8; isin-RU000A101RF5; isin-RU000A102B30; isin-RU000A105FM7; isin-RU000A1074F4; isin-RU000A105SZ2; isin-RU000A1032S5; isin-RU000A103YF7; isin-RU000A105CS1; isin-RU000A1035D0; isin-RU000A105YA3; isin-RU000A106T85; isin-RU000A1057A0; isin-RU000A107EC7; isin-RU000A103RT2; isin-RU000A1034T9; isin-RU000A1064X8; isin-RU000A1021G3; isin-RU000A105Y14; isin-RU000A103H25; isin-RU000A107EW5; isin-RU000A102LW1; isin-RU000A103TV4; isin-RU000A104CJ3; isin-RU000A105GS2; isin-RU000A107761; isin-RU000A104A39</t>
         </is>
       </c>
       <c r="H106" t="inlineStr"/>
@@ -4608,7 +4616,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>no-nbim-24243066d8808900aa83aad2fa3f82386391a8be; no-nbim-cdac1d70dc611fe9778008c596cdbac9bc5aae30; no-nbim-29bd28f22abd51b575faac7f3f4f57516df73a0f; no-nbim-a98688027ef696057436ac536d2806e08f08ce2a; no-nbim-04d3d652aaec156cefc30392e20e9df135838dc6; no-nbim-4c1a5b47ef9e9139d3714247191f7848de77531a; no-nbim-6a2b199890dda3e61e70663d9d061343ed7f0b44; no-nbim-f2711db3ace6b3923197ccbc5ab07c88ab85de6d; no-nbim-1259ddfa74fe8561a65d5568fecbf8fc7d390ce9; no-nbim-e59a37b02764ab08103acda79120d57f92b0e9d8; no-nbim-f7a6fc14e5830607e0d82cc21143bfe98835c1f9; no-nbim-03f813220194494c6f4378503809964840ae59e5; no-nbim-72808d6520e3a318d0311bfe40018ef29abb3b67; no-nbim-3f8405c26d8a9ee2ba4a4fb3a77175463619c6f9; no-nbim-8b6a4bf554175bc617f45779bd74e6b580f48d81; no-nbim-8b87af5e57b0a9582792ce732f36732a8e904e98; no-nbim-c3e7b46c47e084d1f49a6a6f7fdea8afe85f43a0; no-nbim-7c57ff0a0dcc699b19d8ee1c7252d20b2c4080b7; no-nbim-b1367437f1a6c37c53172b26e1b9beabb7cde073; no-nbim-58096145169614c85eefb247eae4f2776439292c; no-nbim-7280750abc4a0ce7f520542cfbc615b38b125b08; no-nbim-18ac276d696774a60180d87f79f22e9ec3e92cd6; no-nbim-488abc09a736121d7e91a31f8bbc2cd7ba70eda0; no-nbim-323e056b6b99094d7b46513044cf7bb6dda21363; no-nbim-b1128c55443c59beacc549745949bba9bc9ca832; no-nbim-ae8bd900e412a004ca50c48a29483cdbfc6c7382; no-nbim-0a21f9d92e5d22044b4008330265e0fc3eda14a8; no-nbim-378eac5fdd03ceb7ba88e2762ec799972edf7e05; no-nbim-6f19cd1f4fad120cd33757084eb0ba0668b2534d; no-nbim-f27c928d32e25ff14143dfaa155709a3f8af6d73; no-nbim-00cd9b92225ae348d3a41182debacd7c675fbdba; no-nbim-6e3d73ce559ae8dc9cb6f017f468fe2cd5183250; no-nbim-7231ea89baba7fe0612495ca66daf4dab0016858; no-nbim-2aba23c8d3974ea46ccc69e2f91fb8f535351988; no-nbim-8dd4ac8c9a64929fa592eac8ecb635ed02ccc012; no-nbim-745f867000cc982938cb62503bf06e54c1b62760; no-nbim-f39839208b0452ed95cd9b2b933e9dba5cd426f6; no-nbim-e6c0bb13870cf1a430085d1effa48e3c64a0770c; no-nbim-5db7361e8217c57bad601198eab0ed42cfa2e113; no-nbim-e46b432878c7e0d42f4d69b67f27481eb4cb26ca</t>
+          <t>no-nbim-b1367437f1a6c37c53172b26e1b9beabb7cde073; no-nbim-03f813220194494c6f4378503809964840ae59e5; no-nbim-6f19cd1f4fad120cd33757084eb0ba0668b2534d; no-nbim-24243066d8808900aa83aad2fa3f82386391a8be; no-nbim-4c1a5b47ef9e9139d3714247191f7848de77531a; no-nbim-e59a37b02764ab08103acda79120d57f92b0e9d8; no-nbim-7280750abc4a0ce7f520542cfbc615b38b125b08; no-nbim-f2711db3ace6b3923197ccbc5ab07c88ab85de6d; no-nbim-f27c928d32e25ff14143dfaa155709a3f8af6d73; no-nbim-7c57ff0a0dcc699b19d8ee1c7252d20b2c4080b7; no-nbim-18ac276d696774a60180d87f79f22e9ec3e92cd6; no-nbim-f39839208b0452ed95cd9b2b933e9dba5cd426f6; no-nbim-f7a6fc14e5830607e0d82cc21143bfe98835c1f9; no-nbim-8dd4ac8c9a64929fa592eac8ecb635ed02ccc012; no-nbim-3f8405c26d8a9ee2ba4a4fb3a77175463619c6f9; no-nbim-e46b432878c7e0d42f4d69b67f27481eb4cb26ca; no-nbim-323e056b6b99094d7b46513044cf7bb6dda21363; no-nbim-378eac5fdd03ceb7ba88e2762ec799972edf7e05; no-nbim-00cd9b92225ae348d3a41182debacd7c675fbdba; no-nbim-745f867000cc982938cb62503bf06e54c1b62760; no-nbim-8b87af5e57b0a9582792ce732f36732a8e904e98; no-nbim-7231ea89baba7fe0612495ca66daf4dab0016858; no-nbim-ae8bd900e412a004ca50c48a29483cdbfc6c7382; no-nbim-b1128c55443c59beacc549745949bba9bc9ca832; no-nbim-a98688027ef696057436ac536d2806e08f08ce2a; no-nbim-c3e7b46c47e084d1f49a6a6f7fdea8afe85f43a0; no-nbim-1259ddfa74fe8561a65d5568fecbf8fc7d390ce9; no-nbim-04d3d652aaec156cefc30392e20e9df135838dc6; no-nbim-8b6a4bf554175bc617f45779bd74e6b580f48d81; no-nbim-6e3d73ce559ae8dc9cb6f017f468fe2cd5183250; no-nbim-72808d6520e3a318d0311bfe40018ef29abb3b67; no-nbim-0a21f9d92e5d22044b4008330265e0fc3eda14a8; no-nbim-6a2b199890dda3e61e70663d9d061343ed7f0b44; no-nbim-2aba23c8d3974ea46ccc69e2f91fb8f535351988; no-nbim-488abc09a736121d7e91a31f8bbc2cd7ba70eda0; no-nbim-58096145169614c85eefb247eae4f2776439292c; no-nbim-e6c0bb13870cf1a430085d1effa48e3c64a0770c; no-nbim-29bd28f22abd51b575faac7f3f4f57516df73a0f; no-nbim-5db7361e8217c57bad601198eab0ed42cfa2e113; no-nbim-cdac1d70dc611fe9778008c596cdbac9bc5aae30</t>
         </is>
       </c>
       <c r="H107" t="inlineStr"/>
@@ -4647,7 +4655,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>isin-RU000A1094U1; isin-RU000A109F05; isin-RU000A109U06; isin-RU000A10AHD7; isin-RU000A10ANT1; isin-RU000A108AC3; isin-RU000A109T41; isin-RU000A109098; isin-RU000A10B7N0; isin-RU000A109RF8; isin-RU000A10B4F3; isin-RU000A109SX9; isin-RU000A10AHU1; isin-RU000A109XN0; isin-RU000A10D7Z2; isin-RU000A109KT4; isin-RU000A10D4S4; isin-RU000A10CT74; isin-RU000A10ABR0; isin-RU000A10CTK3; isin-RU000A108RM6; isin-RU000A10BYZ3; isin-RU000A108ZP2; isin-RU000A109S83; isin-RU000A10BQC8; isin-RU000A108YZ4; isin-RU000A10B2D2; isin-RU000A10BQG9; isin-RU000A10EJR5; isin-RU000A1089A3; isin-RU000A10BVY2; isin-RU000A10BQV8; isin-RU000A10ADR6; isin-RU000A109L49; isin-RU000A108Q78</t>
+          <t>isin-RU000A10B7N0; isin-RU000A109U06; isin-RU000A109RF8; isin-RU000A10ABR0; isin-RU000A10EJR5; isin-RU000A109SX9; isin-RU000A10B2D2; isin-RU000A108ZP2; isin-RU000A1089A3; isin-RU000A109F05; isin-RU000A109KT4; isin-RU000A108Q78; isin-RU000A10BYZ3; isin-RU000A10B4F3; isin-RU000A10AHD7; isin-RU000A10BQV8; isin-RU000A10ANT1; isin-RU000A10BQG9; isin-RU000A108RM6; isin-RU000A108AC3; isin-RU000A10ADR6; isin-RU000A108YZ4; isin-RU000A109L49; isin-RU000A109S83; isin-RU000A10D4S4; isin-RU000A109098; isin-RU000A109XN0; isin-RU000A109T41; isin-RU000A10BQC8; isin-RU000A10AHU1; isin-RU000A10CTK3; isin-RU000A10D7Z2; isin-RU000A10CT74; isin-RU000A1094U1; isin-RU000A10BVY2</t>
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
@@ -4686,7 +4694,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>us-bis-export-addc9eaad7179f57be7289b1ad6cb13813eed376; us-bis-export-214f003a24cdfb02f6e94cab417f141a4b4f5b0f; us-bis-export-68f642482c246dc91a331d362cb8b7d8352b1ccb; us-bis-export-017905e6ca881e90a4e6b614f41816e61ffa48ba; us-bis-export-e09801131ff8870f4e4418de5489263669cc9e85; us-bis-export-67fb9be62a0d9cc537897480269a5c132259bd0e; us-bis-export-fc20e35cd3e3aa6caf7348933f1573ed792ce600; us-bis-export-fd3dd63bbacb452583e792fdc4631bd6cf34d2ed; us-bis-export-f69cee8a19aaead98b1717b4a096e87d9ad83625; us-bis-export-aaebdf3c71a78be66c31dcbe6211d60214de8b61; us-bis-export-e64b37eedd8c2accbaaab47741c503b9fbdab2d9; us-bis-export-15d2dd51273581e9cc181c4346abadee248bcdbb; us-bis-export-cff61b07488f65cd314c507f72c0aa454b493c97; us-bis-export-715a374e32ee019298b1007d7055227517b36c7c; us-bis-export-aa0810be7df98690a0af1cf23781eff12cf25c92; us-bis-export-c651a1aaa4785cd33ebfe7219386c2ba056fd4c4; us-bis-export-72c7352f384bf6c3db45bd897bc249dc39b77ada; us-bis-export-7adf27a15c0879d581a15f8e05368dc22d3da6c9; us-bis-export-72f8a753b6ea15f37ea3f8a1fbeb94b6148e5701; us-bis-export-5b2c46e83495915773d00c93ebb8c29de2c7a2b0; us-bis-export-089c4214fc08b24b46a81c4c933bce3cceb2a983; us-bis-export-398de17a0513103daeab46b698f17e587d81d6c7; us-bis-export-da5bffa6186b357e2e12e02d081e3948a7735d32; us-bis-export-53d825803367590e2ccd23bb0c88d521a0c5d3ea; us-bis-export-4f4bcc6e49ae204f24ee26ff9faecf9482754235; us-bis-export-ff0b6c55f0349af6220392a53dd4e261fe3a2435; us-bis-export-fe6986e7a930fd85f4aa91d6707d01d239239716; us-bis-export-80aebefac84569a5fa588ce4e9cfa2d809645f61; us-bis-export-ffa489e53e4322e29ff62bb29116133a2e640b84; us-bis-export-1018bfb459a547dbd2de6f9e35e1c9cf70f2159f; us-bis-export-3a54f4c0aa1f1c46015a7bcc75ba79fc322cf53b; us-bis-export-0cddfa861dc5fdbca697069e947d0b39cccf3991; us-bis-export-b04a4c7e159c56e5262282b71259e77be2fa39a1; us-bis-export-48d12bddd52d720d8df51e16548342f9e00a422f; us-bis-export-cb0c0836584877297ce648f3c480b2bca54fce27</t>
+          <t>us-bis-export-f69cee8a19aaead98b1717b4a096e87d9ad83625; us-bis-export-715a374e32ee019298b1007d7055227517b36c7c; us-bis-export-addc9eaad7179f57be7289b1ad6cb13813eed376; us-bis-export-ffa489e53e4322e29ff62bb29116133a2e640b84; us-bis-export-72f8a753b6ea15f37ea3f8a1fbeb94b6148e5701; us-bis-export-15d2dd51273581e9cc181c4346abadee248bcdbb; us-bis-export-017905e6ca881e90a4e6b614f41816e61ffa48ba; us-bis-export-214f003a24cdfb02f6e94cab417f141a4b4f5b0f; us-bis-export-fe6986e7a930fd85f4aa91d6707d01d239239716; us-bis-export-398de17a0513103daeab46b698f17e587d81d6c7; us-bis-export-5b2c46e83495915773d00c93ebb8c29de2c7a2b0; us-bis-export-da5bffa6186b357e2e12e02d081e3948a7735d32; us-bis-export-1018bfb459a547dbd2de6f9e35e1c9cf70f2159f; us-bis-export-089c4214fc08b24b46a81c4c933bce3cceb2a983; us-bis-export-e09801131ff8870f4e4418de5489263669cc9e85; us-bis-export-aaebdf3c71a78be66c31dcbe6211d60214de8b61; us-bis-export-c651a1aaa4785cd33ebfe7219386c2ba056fd4c4; us-bis-export-67fb9be62a0d9cc537897480269a5c132259bd0e; us-bis-export-cb0c0836584877297ce648f3c480b2bca54fce27; us-bis-export-aa0810be7df98690a0af1cf23781eff12cf25c92; us-bis-export-ff0b6c55f0349af6220392a53dd4e261fe3a2435; us-bis-export-0cddfa861dc5fdbca697069e947d0b39cccf3991; us-bis-export-b04a4c7e159c56e5262282b71259e77be2fa39a1; us-bis-export-72c7352f384bf6c3db45bd897bc249dc39b77ada; us-bis-export-48d12bddd52d720d8df51e16548342f9e00a422f; us-bis-export-80aebefac84569a5fa588ce4e9cfa2d809645f61; us-bis-export-53d825803367590e2ccd23bb0c88d521a0c5d3ea; us-bis-export-68f642482c246dc91a331d362cb8b7d8352b1ccb; us-bis-export-e64b37eedd8c2accbaaab47741c503b9fbdab2d9; us-bis-export-3a54f4c0aa1f1c46015a7bcc75ba79fc322cf53b; us-bis-export-cff61b07488f65cd314c507f72c0aa454b493c97; us-bis-export-fc20e35cd3e3aa6caf7348933f1573ed792ce600; us-bis-export-fd3dd63bbacb452583e792fdc4631bd6cf34d2ed; us-bis-export-4f4bcc6e49ae204f24ee26ff9faecf9482754235; us-bis-export-7adf27a15c0879d581a15f8e05368dc22d3da6c9</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -4725,7 +4733,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>isin-MD0000000108; isin-MD00000001J5; isin-MD0000000140; isin-MD00000000T6; isin-MD00000000W0; isin-MD00000001D8; isin-MD0000000181; isin-MD00000001G1; isin-MD00000000Q2; isin-MD00000000N9; isin-MD00000000P4; isin-MD0000000165; isin-MD00000001A4; isin-MD0000000116; isin-MD00000000V2; isin-MD0000000132; isin-MD00000000S8; isin-MD00000000X8; isin-MD00000001C0; isin-MD00000000R0; isin-MD00000000M1; isin-MD00000001H9; isin-MD00000000U4; isin-MD0000000173; isin-MD00000001F3; isin-MD00000001B2; isin-MD00000001K3; isin-MD0000000124; isin-MD0000000157; isin-MD00000001E6; isin-MD00000000Z3; isin-MD0000000199; isin-MD00000000Y6</t>
+          <t>isin-MD00000000X8; isin-MD00000000Y6; isin-MD0000000157; isin-MD00000001H9; isin-MD00000001F3; isin-MD00000000P4; isin-MD00000001D8; isin-MD0000000116; isin-MD00000000Z3; isin-MD0000000108; isin-MD0000000199; isin-MD00000000R0; isin-MD0000000181; isin-MD0000000132; isin-MD00000001E6; isin-MD00000001G1; isin-MD0000000124; isin-MD00000000Q2; isin-MD00000000M1; isin-MD00000000S8; isin-MD00000001K3; isin-MD00000000T6; isin-MD0000000165; isin-MD00000001B2; isin-MD0000000140; isin-MD00000000V2; isin-MD00000000U4; isin-MD00000001J5; isin-MD00000001C0; isin-MD0000000173; isin-MD00000000N9; isin-MD00000000W0; isin-MD00000001A4</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -4764,7 +4772,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>us-bis-export-a0ccfd123bf8cc372b9134176df810f1c760ef54; us-bis-export-7e189a7e488822a4c1554f0474013861621bce61; us-bis-export-bcf1cd55b6a04526b5fd75dcd526a39f323d9387; us-bis-export-301fd5f060900e2224fa455052547bb1694513de; us-bis-export-73dc8e9c4cb57e4de4a8fe96d0118eeae00d8617; us-bis-export-06bb0a79def0ef22e344fdbd504bfeb1ce0dfe4a; us-bis-export-ffe0df675b44752d79dc997052d0fbfe1e93979f; us-bis-export-31f7d5711f771edc5006c21468c587539af67120; us-bis-export-a9fc187c0be07e688652ce2cf5f87d7f93bbc19a; us-bis-export-92748483e3b0f4e0b74b4c4b674aedb71d15ed6f; us-bis-export-940a74de0548faef86a2558abdc06808bdcdd325; us-bis-export-4fa60884e751c73b6644ee582fa06fab6f90ffaa; us-bis-export-983c71596a66e17f9f014b74b251fb274dbcfc8c; us-bis-export-31f361cc0390b229ad15bea91b071dcc5de6dd90; us-bis-export-b949a1aced01a5ceac0b4d5a3af1bc2ce495ba98; us-bis-export-27d191f5b81119c5f709a3ac40d40c7959f006a6; us-bis-export-815509e0754998f325e7738d9889f1f309ef58af; us-bis-export-b26be92e21c8c1d9466e438b753fb8c1253706c5; us-bis-export-c6cf3e802d69999e3e468b98de6ae9782a952e2f; us-bis-export-bcd168d2e45968950cdc7f993ea6c2fa4e1119b4; us-bis-export-6f42780a26246d310b4d0ea598214d4a3e962766; us-bis-export-e24e38dfa01950f2b8a80030db095ec0082df0e8; us-bis-export-2a4ee3d6809f07c16d71aff66747c090e0bccec8; us-bis-export-88602ee629430a369cb009335d124599cb3f156d; us-bis-export-3da8479afaffe46a28787d3da8e77ac121c82cbb; us-bis-export-2431f0791bdc64b4ed4a8153303bf5852174987b; us-bis-export-d55836d80b606eb7a271e482b28cec8e7aacff93; us-bis-export-03a23ae39a5008dd9c442562dabebe478398990c; us-bis-export-3fb735923314992d912c21e90622d82f347395f9; us-bis-export-0d60a0eb7d57a2f8f47629f59be30ecdb1931910; us-bis-export-bf5a966121434970439120344a45d42244cc287e; us-bis-export-44be864c9ad2512a200a2fe7f631e2b08312b19f</t>
+          <t>us-bis-export-7e189a7e488822a4c1554f0474013861621bce61; us-bis-export-6f42780a26246d310b4d0ea598214d4a3e962766; us-bis-export-d55836d80b606eb7a271e482b28cec8e7aacff93; us-bis-export-983c71596a66e17f9f014b74b251fb274dbcfc8c; us-bis-export-06bb0a79def0ef22e344fdbd504bfeb1ce0dfe4a; us-bis-export-2431f0791bdc64b4ed4a8153303bf5852174987b; us-bis-export-44be864c9ad2512a200a2fe7f631e2b08312b19f; us-bis-export-03a23ae39a5008dd9c442562dabebe478398990c; us-bis-export-3fb735923314992d912c21e90622d82f347395f9; us-bis-export-73dc8e9c4cb57e4de4a8fe96d0118eeae00d8617; us-bis-export-b949a1aced01a5ceac0b4d5a3af1bc2ce495ba98; us-bis-export-bf5a966121434970439120344a45d42244cc287e; us-bis-export-e24e38dfa01950f2b8a80030db095ec0082df0e8; us-bis-export-2a4ee3d6809f07c16d71aff66747c090e0bccec8; us-bis-export-4fa60884e751c73b6644ee582fa06fab6f90ffaa; us-bis-export-88602ee629430a369cb009335d124599cb3f156d; us-bis-export-bcd168d2e45968950cdc7f993ea6c2fa4e1119b4; us-bis-export-c6cf3e802d69999e3e468b98de6ae9782a952e2f; us-bis-export-31f361cc0390b229ad15bea91b071dcc5de6dd90; us-bis-export-0d60a0eb7d57a2f8f47629f59be30ecdb1931910; us-bis-export-a0ccfd123bf8cc372b9134176df810f1c760ef54; us-bis-export-a9fc187c0be07e688652ce2cf5f87d7f93bbc19a; us-bis-export-31f7d5711f771edc5006c21468c587539af67120; us-bis-export-b26be92e21c8c1d9466e438b753fb8c1253706c5; us-bis-export-ffe0df675b44752d79dc997052d0fbfe1e93979f; us-bis-export-815509e0754998f325e7738d9889f1f309ef58af; us-bis-export-92748483e3b0f4e0b74b4c4b674aedb71d15ed6f; us-bis-export-301fd5f060900e2224fa455052547bb1694513de; us-bis-export-bcf1cd55b6a04526b5fd75dcd526a39f323d9387; us-bis-export-3da8479afaffe46a28787d3da8e77ac121c82cbb; us-bis-export-27d191f5b81119c5f709a3ac40d40c7959f006a6; us-bis-export-940a74de0548faef86a2558abdc06808bdcdd325</t>
         </is>
       </c>
       <c r="H111" t="inlineStr"/>
@@ -4803,7 +4811,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>us-bis-export-f99313b649d12e4ccae17071aeccfee9b2631eeb; us-bis-export-b2bd96ae85c35a3f9751b34c881f017a6eb1f0e0; us-bis-export-f12307bf48e679aad730086ec0b61fa7b69a6284; us-bis-export-fa39e47b91c1c90eade87fd8b67a2d7972e96aec; us-bis-export-d6ec79f11520eae93b93462fd847b11e1d72bf17; us-bis-export-ef1183c391fa262a91b4e73be4fc0cd67b4948fb; us-bis-export-51b2e4e85ff629d1c3e456dec6d9f573d6ed6170; us-bis-export-90bc1c356cd2a51a1a97fe05e282732f8348f015; us-bis-export-488c38fe4ce0d8d151804c0c7549084bdafae9cd; us-bis-export-7a7db7f27d843f1d169217e393e41d2f0bde84ac; us-bis-export-6b106cf13ccb9fd8815bfaa6996016e4fc857ad3; us-bis-export-11787cb69f7a602f005bef26ae3349973eb7060b; us-bis-export-955fea2f9fb09617dda89b7528c773f14580990d; us-bis-export-ddcf913041bce9f96b2cc2466b9f02b1bd063c1e; us-bis-export-80b852d2c75f4cc0ab0acce03004223141a2eeb9; us-bis-export-c502ecf6d529ee0254d8ac7d265dd1490cf6ab9b; us-bis-export-b4d96d2f9caa77a03d23b9b4a473f52ab22acb31; us-bis-export-9847035a4242a1c67459f37cb2c06ada021324a4; us-bis-export-a9e84cb9b949de92ebfd16c886b9f605e878f4db; us-bis-export-72de6bd48d0053431c9dd42bcf09f430b2f99b05; us-bis-export-2ac84fa5eb1bdda9761c6023570852144036a326; us-bis-export-91789ce0d07d33dddd8b4d5cb9bc9b9db4f74f13; us-bis-export-1cef5f66404333a52a94b912423647c9b75b34f6; us-bis-export-b9055cb42114695988163440d36f8721c9002869; us-bis-export-8a01baf8766fb7992d3cbe4409af6c640da98ced; us-bis-export-5bf8e4ecd7e131917e72b6ef0883929aa373564c; us-bis-export-4ce440334e69c64c29963b028b8b97b2c3fa802a; us-bis-export-415c2bcdf7a09e593791cd9a81972970d66e054b; us-bis-export-e2140c02fdd068e95baf3f050a892b5524004c4f; us-bis-export-759ffef9195d76d4a25aa9a2e32cf840679ae8a4; us-bis-export-2b220cadc3050cc042a8f9fa68e0156a8efb2007; us-bis-export-a6a1dc9f781c40d887dc717159b449d53525fe74</t>
+          <t>us-bis-export-b9055cb42114695988163440d36f8721c9002869; us-bis-export-955fea2f9fb09617dda89b7528c773f14580990d; us-bis-export-f12307bf48e679aad730086ec0b61fa7b69a6284; us-bis-export-415c2bcdf7a09e593791cd9a81972970d66e054b; us-bis-export-91789ce0d07d33dddd8b4d5cb9bc9b9db4f74f13; us-bis-export-ddcf913041bce9f96b2cc2466b9f02b1bd063c1e; us-bis-export-5bf8e4ecd7e131917e72b6ef0883929aa373564c; us-bis-export-8a01baf8766fb7992d3cbe4409af6c640da98ced; us-bis-export-d6ec79f11520eae93b93462fd847b11e1d72bf17; us-bis-export-11787cb69f7a602f005bef26ae3349973eb7060b; us-bis-export-4ce440334e69c64c29963b028b8b97b2c3fa802a; us-bis-export-90bc1c356cd2a51a1a97fe05e282732f8348f015; us-bis-export-b4d96d2f9caa77a03d23b9b4a473f52ab22acb31; us-bis-export-b2bd96ae85c35a3f9751b34c881f017a6eb1f0e0; us-bis-export-488c38fe4ce0d8d151804c0c7549084bdafae9cd; us-bis-export-9847035a4242a1c67459f37cb2c06ada021324a4; us-bis-export-759ffef9195d76d4a25aa9a2e32cf840679ae8a4; us-bis-export-c502ecf6d529ee0254d8ac7d265dd1490cf6ab9b; us-bis-export-7a7db7f27d843f1d169217e393e41d2f0bde84ac; us-bis-export-6b106cf13ccb9fd8815bfaa6996016e4fc857ad3; us-bis-export-a9e84cb9b949de92ebfd16c886b9f605e878f4db; us-bis-export-a6a1dc9f781c40d887dc717159b449d53525fe74; us-bis-export-80b852d2c75f4cc0ab0acce03004223141a2eeb9; us-bis-export-ef1183c391fa262a91b4e73be4fc0cd67b4948fb; us-bis-export-e2140c02fdd068e95baf3f050a892b5524004c4f; us-bis-export-2ac84fa5eb1bdda9761c6023570852144036a326; us-bis-export-51b2e4e85ff629d1c3e456dec6d9f573d6ed6170; us-bis-export-2b220cadc3050cc042a8f9fa68e0156a8efb2007; us-bis-export-fa39e47b91c1c90eade87fd8b67a2d7972e96aec; us-bis-export-1cef5f66404333a52a94b912423647c9b75b34f6; us-bis-export-f99313b649d12e4ccae17071aeccfee9b2631eeb; us-bis-export-72de6bd48d0053431c9dd42bcf09f430b2f99b05</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -4842,7 +4850,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>isin-RU000A104BU2; isin-RU000A107225; isin-RU000A1074E7; isin-RU000A105BW5; isin-RU000A106VN0; isin-RU000A103WD6; isin-RU000A1032D7; isin-RU000A106YD5; isin-RU000A107BD1; isin-RU000A105AX5; isin-RU000A101PV6; isin-RU000A104W82; isin-RU000A107PE9; isin-RU000A104V59; isin-RU000A104UY4; isin-RU000A106TJ2; isin-RU000A107DD7; isin-RU000A105RU5; isin-RU000A106W49; isin-RU000A104WZ7; isin-RU000A1049M2; isin-RU000A103FT7; isin-RU000A102580; isin-RU000A106ZZ5; isin-RU000A1053W3; isin-RU000A104A05; isin-RU000A103G83; isin-RU000A105VP7; isin-RU000A107G63; isin-RU000A104C78; isin-RU000A105ZF9</t>
+          <t>isin-RU000A103FT7; isin-RU000A104V59; isin-RU000A106VN0; isin-RU000A1032D7; isin-RU000A106YD5; isin-RU000A107PE9; isin-RU000A107225; isin-RU000A104A05; isin-RU000A1074E7; isin-RU000A106W49; isin-RU000A107DD7; isin-RU000A103G83; isin-RU000A104WZ7; isin-RU000A101PV6; isin-RU000A103WD6; isin-RU000A107G63; isin-RU000A1053W3; isin-RU000A104W82; isin-RU000A106ZZ5; isin-RU000A104BU2; isin-RU000A102580; isin-RU000A105AX5; isin-RU000A104UY4; isin-RU000A1049M2; isin-RU000A104C78; isin-RU000A107BD1; isin-RU000A105ZF9; isin-RU000A105RU5; isin-RU000A106TJ2; isin-RU000A105BW5; isin-RU000A105VP7</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
@@ -4881,7 +4889,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>isin-RU000A105EP3; isin-RU000A105LS2; isin-RU000A108462; isin-RU000A106GC4; isin-RU000A1051U1; isin-RU000A103604; isin-RU000A107LU4; isin-RU000A105YB1; isin-RU000A103RY2; isin-RU000A1057D4; isin-RU000A1046N6; isin-RU000A102AB8; isin-RU000A106AK0; isin-RU000A104G90; isin-RU000A107AZ6; isin-RU000A106CB5; isin-RU000A106U74; isin-RU000A1079G1; isin-RU000A101UR4; isin-RU000A107548; isin-RU000A106XJ4; isin-RU000A101RH1; isin-RU000A1034J0; isin-RU000A106HB4; isin-RU000A107E08; isin-RU000A105JG1; isin-RU000A102TR4; isin-RU000A106A86; isin-RU000A104CK1; isin-RU000A109QN4; isin-RU000A1061L9</t>
+          <t>isin-RU000A105JG1; isin-RU000A104CK1; isin-RU000A106HB4; isin-RU000A108462; isin-RU000A1034J0; isin-RU000A106U74; isin-RU000A105LS2; isin-RU000A103RY2; isin-RU000A1051U1; isin-RU000A1057D4; isin-RU000A107LU4; isin-RU000A106AK0; isin-RU000A103604; isin-RU000A101RH1; isin-RU000A1046N6; isin-RU000A1079G1; isin-RU000A105EP3; isin-RU000A102TR4; isin-RU000A106GC4; isin-RU000A107548; isin-RU000A106CB5; isin-RU000A106XJ4; isin-RU000A107E08; isin-RU000A105YB1; isin-RU000A104G90; isin-RU000A106A86; isin-RU000A107AZ6; isin-RU000A102AB8; isin-RU000A101UR4; isin-RU000A109QN4; isin-RU000A1061L9</t>
         </is>
       </c>
       <c r="H114" t="inlineStr"/>
@@ -4920,7 +4928,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>isin-RU000A10BJL4; isin-RU000A10B0R6; isin-RU000A107YT9; isin-RU000A1098H9; isin-RU000A10AYB6; isin-RU000A108ZQ0; isin-RU000A10EL13; isin-RU000A10BU72; isin-RU000A10B1X2; isin-RU000A10AGA5; isin-RU000A10EK63; isin-RU000A10D665; isin-RU000A10AHJ4; isin-RU000A109SM2; isin-RU000A10CU30; isin-RU000A10AA02; isin-RU000A109KV0; isin-RU000A10AZG2; isin-RU000A10ECR0; isin-RU000A109SH2; isin-RU000A10C8H9; isin-RU000A10E9V6; isin-RU000A10A9K3; isin-RU000A1086N2; isin-RU000A108G70; isin-RU000A10B255; isin-RU000A10B7W1; isin-RU000A107T76; isin-RU000A10DMN0; isin-RU000A10A7H3; isin-RU000A10BWA0</t>
+          <t>isin-RU000A10EK63; isin-RU000A10AZG2; isin-RU000A10A9K3; isin-RU000A10AYB6; isin-RU000A109SH2; isin-RU000A10E9V6; isin-RU000A10ECR0; isin-RU000A10B0R6; isin-RU000A10CU30; isin-RU000A109SM2; isin-RU000A10BJL4; isin-RU000A1098H9; isin-RU000A1086N2; isin-RU000A10EL13; isin-RU000A10AGA5; isin-RU000A10BU72; isin-RU000A109KV0; isin-RU000A10C8H9; isin-RU000A10BWA0; isin-RU000A108ZQ0; isin-RU000A107T76; isin-RU000A10B1X2; isin-RU000A10D665; isin-RU000A10A7H3; isin-RU000A10DMN0; isin-RU000A10AHJ4; isin-RU000A108G70; isin-RU000A10B255; isin-RU000A10B7W1; isin-RU000A10AA02; isin-RU000A107YT9</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -4959,7 +4967,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>us-bis-export-82946210a8ddd470012f452ceae625c911696185; us-bis-export-a436233d2c6c56d960ebeb75515ff472269af881; us-bis-export-35b933a4c0b21fb19e559d4e0dbf8eb803f7736e; us-bis-export-2424eac5562e3affcd5d3bffd15bddf88174ccc6; us-bis-export-f9fefa36e1f866d630ded91684f83a1b6706930d; us-bis-export-1f6b4cd4b222a77730cdc398d633455b1f54f068; us-bis-export-cbb6d8ecb514e3ae89dcaa1ad8ca4e0f4a1d3a8c; us-bis-export-a26010f4fbdff031cfbdd506b0c5473ba960de7c; us-bis-export-b567ef733ad59c447f4c37a0517c908ecaccb1a3; us-bis-export-7f2bd212278962a3422ea337f4a3c48d89b32dd5; us-bis-export-9544416209657983bc7001b37e9d51060e72c975; us-bis-export-8f3a6f47d9a111ce430642008abc33d24ae2de0e; us-bis-export-dcceee15992199faf14eaa560e50eed1ac08cbff; us-bis-export-76c90086df375e179d659f91819baed6c68924e5; us-bis-export-40cd785444939a13431fc3c0043e48fb491a19eb; us-bis-export-c898c0d259425509cbcff7d87255626129febe27; us-bis-export-451dbff38586313accead9604ed19a829c697a0c; us-bis-export-9fca9bb2f6eb7b7731bc17f0bfdbe5357d71b549; us-bis-export-f406edccfacbefd295d97789ad1f04d4be950e5f; us-bis-export-304a2d6acccb011ca183d5f74eb09e2adb1b3f7a; us-bis-export-6fc4f02e29c3ce6946bba5ab46d85e6ddbd52011; us-bis-export-c273c16bf1303dd4a5ff63495ce04d48fb684bc8; us-bis-export-d07aa04f8fddc24521918cbd3fa708a9aff6b70f; us-bis-export-d6ace3d53c1f5a32f9b42d5191ab03efb00ca334; us-bis-export-db7e4415c40f144b86ae7e80663f1ecb3881c3f0; us-bis-export-5cea7d6d73036aed3a9b84b3acbf2ab4da5a5894; us-bis-export-62390dd00f64cd145f6da993b7584bc6576bbc59; us-bis-export-1a9181e9257e6781077da912c08bb91341bf776c; us-bis-export-1878696a0dfcc2b4df8fe4c1b4c18ea191d2379a; us-bis-export-429c02d458e26a3481e118ac2c5c839067149dcb; us-bis-export-a5e2916444556c0a92de66fe972dfc4267458783</t>
+          <t>us-bis-export-429c02d458e26a3481e118ac2c5c839067149dcb; us-bis-export-76c90086df375e179d659f91819baed6c68924e5; us-bis-export-1878696a0dfcc2b4df8fe4c1b4c18ea191d2379a; us-bis-export-7f2bd212278962a3422ea337f4a3c48d89b32dd5; us-bis-export-6fc4f02e29c3ce6946bba5ab46d85e6ddbd52011; us-bis-export-b567ef733ad59c447f4c37a0517c908ecaccb1a3; us-bis-export-82946210a8ddd470012f452ceae625c911696185; us-bis-export-2424eac5562e3affcd5d3bffd15bddf88174ccc6; us-bis-export-9fca9bb2f6eb7b7731bc17f0bfdbe5357d71b549; us-bis-export-5cea7d6d73036aed3a9b84b3acbf2ab4da5a5894; us-bis-export-304a2d6acccb011ca183d5f74eb09e2adb1b3f7a; us-bis-export-a26010f4fbdff031cfbdd506b0c5473ba960de7c; us-bis-export-c273c16bf1303dd4a5ff63495ce04d48fb684bc8; us-bis-export-1a9181e9257e6781077da912c08bb91341bf776c; us-bis-export-62390dd00f64cd145f6da993b7584bc6576bbc59; us-bis-export-f9fefa36e1f866d630ded91684f83a1b6706930d; us-bis-export-d07aa04f8fddc24521918cbd3fa708a9aff6b70f; us-bis-export-40cd785444939a13431fc3c0043e48fb491a19eb; us-bis-export-f406edccfacbefd295d97789ad1f04d4be950e5f; us-bis-export-451dbff38586313accead9604ed19a829c697a0c; us-bis-export-c898c0d259425509cbcff7d87255626129febe27; us-bis-export-a436233d2c6c56d960ebeb75515ff472269af881; us-bis-export-db7e4415c40f144b86ae7e80663f1ecb3881c3f0; us-bis-export-35b933a4c0b21fb19e559d4e0dbf8eb803f7736e; us-bis-export-d6ace3d53c1f5a32f9b42d5191ab03efb00ca334; us-bis-export-dcceee15992199faf14eaa560e50eed1ac08cbff; us-bis-export-cbb6d8ecb514e3ae89dcaa1ad8ca4e0f4a1d3a8c; us-bis-export-1f6b4cd4b222a77730cdc398d633455b1f54f068; us-bis-export-9544416209657983bc7001b37e9d51060e72c975; us-bis-export-8f3a6f47d9a111ce430642008abc33d24ae2de0e; us-bis-export-a5e2916444556c0a92de66fe972dfc4267458783</t>
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
@@ -4998,7 +5006,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>isin-RU000A106VR1; isin-RU000A102R32; isin-RU000A107D82; isin-RU000A105X15; isin-RU000A102U11; isin-RU000A106482; isin-RU000A103S55; isin-RU000A104UG1; isin-RU000A1022A4; isin-RU000A105Q14; isin-RU000A103UF5; isin-RU000A103DD6; isin-RU000A107FF7; isin-RU000A102VH1; isin-RU000A1075B0; isin-RU000A101W10; isin-RU000A103075; isin-RU000A106L83; isin-RU000A103B88; isin-RU000A102L46; isin-RU000A102X34; isin-RU000A1085E3; isin-RU000A102440; isin-RU000A106HD0; isin-RU000A1089S5; isin-RU000A101K55; isin-RU000A1086L6; isin-RU000A1026K4; isin-RU000A102TX2; isin-RU000A107H88</t>
+          <t>isin-RU000A101W10; isin-RU000A103DD6; isin-RU000A1026K4; isin-RU000A101K55; isin-RU000A102R32; isin-RU000A102X34; isin-RU000A103075; isin-RU000A103B88; isin-RU000A102U11; isin-RU000A103S55; isin-RU000A105X15; isin-RU000A103UF5; isin-RU000A102VH1; isin-RU000A102L46; isin-RU000A1089S5; isin-RU000A1075B0; isin-RU000A102TX2; isin-RU000A107D82; isin-RU000A106482; isin-RU000A106HD0; isin-RU000A106VR1; isin-RU000A1085E3; isin-RU000A102440; isin-RU000A107H88; isin-RU000A105Q14; isin-RU000A107FF7; isin-RU000A104UG1; isin-RU000A1086L6; isin-RU000A1022A4; isin-RU000A106L83</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
@@ -5037,7 +5045,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>us-bis-export-01ae5f53cb8631efd22c90634e6b3f0daf2b31f4; us-bis-export-383cff5848ac7f218f43781e941b0138efe4f0a6; us-bis-export-57dea62331f8c2e7af9b5625b136ff9862259408; us-bis-export-a81c6ecf08dc8f41ea6ba548054e8b87e9b97b43; us-bis-export-6730408c0d53c0074ee6156b980c3c96a4de249e; us-bis-export-6b68e59a1ea2c1e4fc58700e0e539bf48fd569e7; us-bis-export-fb77edb924adb6876a9eb963e1fee728d0f26d29; us-bis-export-ee6a6e5af365fdab9dfdf4382496f828293787b8; us-bis-export-a62f88117e7a420904e2b0a06c4e7b256c594e52; us-bis-export-56cd1b244736bd025ae02ba2bb3c42cf4f733360; us-bis-export-2b378b31be5be3d7cfe08ef29e5b894c837ccb86; us-bis-export-50cc107b01da267da5a31d838e32cc3d4c65c52e; us-bis-export-56c858a23bf62b610bbbcfbd8a7b78895c04579b; us-bis-export-8c51d1e6c48e218a993a6720102d00df4e2408ec; us-bis-export-fec8679ca8682155494c6534a4ee5b21ff3b7f9d; us-bis-export-4b8628aefdd6624df65a4477ea628b9f3a2af0b4; us-bis-export-65ba375c8e6f9e21c9f8362aeb4153162ecf0fa3; us-bis-export-624b97a8603a7ef546c92a35c4d3e5af1d3cc876; us-bis-export-cadaadb3ac5e8ef7a86f871335e4c2fdf76cd4c4; us-bis-export-7d393aff5c5b87ee72a9545b088f8d98844d68c2; us-bis-export-f4ff7f96cc5933c7c792a69eb76f13e6d555276f; us-bis-export-7463531a400c15127b969e23180cf9a82edb5cb6; us-bis-export-7b39486b819d36e8a9aa6fd1d68825ebfcb30458; us-bis-export-ca88d5cb40a7fa4b0250bbc0b73836a3adf91e53; us-bis-export-6201250cfe17b557bda528f743f53f9049a438a8; us-bis-export-9a6860735e4fe52c2be61d3c2a950cb1ab0f3e2d; us-bis-export-c3784bbfd503e94dc14dec4604a7db7fea3a286b; us-bis-export-f393a6b2d87c456e8d74cc3269c4e3ee7e7e6ee8; us-bis-export-410c573386c9014d71542333965e0712707af209; us-bis-export-06828ca4f4352159d0852bc986b8c3f289ef3f51</t>
+          <t>us-bis-export-7b39486b819d36e8a9aa6fd1d68825ebfcb30458; us-bis-export-c3784bbfd503e94dc14dec4604a7db7fea3a286b; us-bis-export-2b378b31be5be3d7cfe08ef29e5b894c837ccb86; us-bis-export-06828ca4f4352159d0852bc986b8c3f289ef3f51; us-bis-export-f393a6b2d87c456e8d74cc3269c4e3ee7e7e6ee8; us-bis-export-4b8628aefdd6624df65a4477ea628b9f3a2af0b4; us-bis-export-7d393aff5c5b87ee72a9545b088f8d98844d68c2; us-bis-export-a81c6ecf08dc8f41ea6ba548054e8b87e9b97b43; us-bis-export-57dea62331f8c2e7af9b5625b136ff9862259408; us-bis-export-01ae5f53cb8631efd22c90634e6b3f0daf2b31f4; us-bis-export-6b68e59a1ea2c1e4fc58700e0e539bf48fd569e7; us-bis-export-ee6a6e5af365fdab9dfdf4382496f828293787b8; us-bis-export-50cc107b01da267da5a31d838e32cc3d4c65c52e; us-bis-export-fec8679ca8682155494c6534a4ee5b21ff3b7f9d; us-bis-export-56c858a23bf62b610bbbcfbd8a7b78895c04579b; us-bis-export-9a6860735e4fe52c2be61d3c2a950cb1ab0f3e2d; us-bis-export-65ba375c8e6f9e21c9f8362aeb4153162ecf0fa3; us-bis-export-cadaadb3ac5e8ef7a86f871335e4c2fdf76cd4c4; us-bis-export-383cff5848ac7f218f43781e941b0138efe4f0a6; us-bis-export-6730408c0d53c0074ee6156b980c3c96a4de249e; us-bis-export-8c51d1e6c48e218a993a6720102d00df4e2408ec; us-bis-export-6201250cfe17b557bda528f743f53f9049a438a8; us-bis-export-ca88d5cb40a7fa4b0250bbc0b73836a3adf91e53; us-bis-export-7463531a400c15127b969e23180cf9a82edb5cb6; us-bis-export-624b97a8603a7ef546c92a35c4d3e5af1d3cc876; us-bis-export-fb77edb924adb6876a9eb963e1fee728d0f26d29; us-bis-export-f4ff7f96cc5933c7c792a69eb76f13e6d555276f; us-bis-export-a62f88117e7a420904e2b0a06c4e7b256c594e52; us-bis-export-56cd1b244736bd025ae02ba2bb3c42cf4f733360; us-bis-export-410c573386c9014d71542333965e0712707af209</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -5076,7 +5084,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>us-bis-export-7b8d4306cbdf967e6b1418ff9b8d7cbbf2487f3f; us-bis-export-a64597da05d34f192cf95bcb90fb58e6cac1652f; us-bis-export-4e109e82fe18d47620c00dc09394a4ef4ed9da71; us-bis-export-706620519ae8fb4a4f810db388260dd30a726c8e; us-bis-export-818e037bb2ded176db067dc33676e2a3f4d8f743; us-bis-export-9e62fb0688a129e7e96b9dff2d17b58b212f0f01; us-bis-export-b4c8aa4ca313e77b4d9ed20daa9c74bc9bd0cc53; us-bis-export-c3323518637a543be9fac0aab0cdc6ae8efd7814; us-bis-export-c1e49f54dbce7c0453458badad6ac55f0021cffd; us-bis-export-264ec488b29d10deb039c247b8496208b7397ace; us-bis-export-36009800af7c39398369bfb9bb81d15a0b3db475; us-bis-export-11c361b6153227df3d2e88a538cb8e1c38781e10; us-bis-export-82548c7060d832ddd7882f64487d9a448f17842d; us-bis-export-b6a264525172d04cd3d2b4609777b90358477b43; us-bis-export-4f57f38b7f9f60b8ef3808c3860f840fef4debdc; us-bis-export-26d6fe1a73312236b6ad7548adea92b51141da62; us-bis-export-e0218cee700092b2f6e9e01f38f88166dec80343; us-bis-export-647c6830d2826b8cd845c42a5eae9946429bdc86; us-bis-export-5c477c9119a9029785a81caaffd8b312366bb263; us-bis-export-5c00d8e1a29d0ae4c3146ad227436b1eb4f6450a; us-bis-export-39df58af4c9b98953a93b20e4717f44a671de9be; us-bis-export-21af2fdba43d96b925a0f037798cfbf6210e125c; us-bis-export-feaf8da9b888e9080c6e4b361159ee272edb8798; us-bis-export-29286f39362e16186ff66f43d824d7c149d0cf5e; us-bis-export-4264a0e89e0393d46b2582026729a197345799b6; us-bis-export-a83c03e85a008168cf2e0f6dd76eb708a5ae0197; us-bis-export-f12a0e20903f165eca9af99697055b33105a9736; us-bis-export-39a6126126def4ea71a8893ca31d8ed2ddea624e</t>
+          <t>us-bis-export-9e62fb0688a129e7e96b9dff2d17b58b212f0f01; us-bis-export-264ec488b29d10deb039c247b8496208b7397ace; us-bis-export-a83c03e85a008168cf2e0f6dd76eb708a5ae0197; us-bis-export-29286f39362e16186ff66f43d824d7c149d0cf5e; us-bis-export-4f57f38b7f9f60b8ef3808c3860f840fef4debdc; us-bis-export-7b8d4306cbdf967e6b1418ff9b8d7cbbf2487f3f; us-bis-export-36009800af7c39398369bfb9bb81d15a0b3db475; us-bis-export-4e109e82fe18d47620c00dc09394a4ef4ed9da71; us-bis-export-a64597da05d34f192cf95bcb90fb58e6cac1652f; us-bis-export-c1e49f54dbce7c0453458badad6ac55f0021cffd; us-bis-export-11c361b6153227df3d2e88a538cb8e1c38781e10; us-bis-export-c3323518637a543be9fac0aab0cdc6ae8efd7814; us-bis-export-5c477c9119a9029785a81caaffd8b312366bb263; us-bis-export-4264a0e89e0393d46b2582026729a197345799b6; us-bis-export-39a6126126def4ea71a8893ca31d8ed2ddea624e; us-bis-export-5c00d8e1a29d0ae4c3146ad227436b1eb4f6450a; us-bis-export-21af2fdba43d96b925a0f037798cfbf6210e125c; us-bis-export-feaf8da9b888e9080c6e4b361159ee272edb8798; us-bis-export-b6a264525172d04cd3d2b4609777b90358477b43; us-bis-export-818e037bb2ded176db067dc33676e2a3f4d8f743; us-bis-export-647c6830d2826b8cd845c42a5eae9946429bdc86; us-bis-export-f12a0e20903f165eca9af99697055b33105a9736; us-bis-export-39df58af4c9b98953a93b20e4717f44a671de9be; us-bis-export-706620519ae8fb4a4f810db388260dd30a726c8e; us-bis-export-b4c8aa4ca313e77b4d9ed20daa9c74bc9bd0cc53; us-bis-export-26d6fe1a73312236b6ad7548adea92b51141da62; us-bis-export-e0218cee700092b2f6e9e01f38f88166dec80343; us-bis-export-82548c7060d832ddd7882f64487d9a448f17842d</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -5115,7 +5123,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>us-occ-21610-first-national-bank; us-occ-11968-first-national-bank; us-occ-20214-first-national-bank; NK-RPrxx7QDMC48WoRtfsVSYZ; us-occ-10230-first-national-bank; us-occ-17324-first-national-bank; us-occ-12423-first-national-bank; NK-VEUcR2WqX6PU6EAJe9248K; NK-hNd7gSkdsgEtc2Cu2ehWpY; us-occ-7853-first-national-bank; us-occ-14163-first-national-bank; us-occ-14012-first-national-bank; us-occ-17129-first-national-bank; us-occ-3496-first-national-bank; NK-aHpDcBPsCBsGiDs3VB9FMV; NK-PQKV6m5qiHTwLDWU7iXqBn; us-occ-13830-first-national-bank; us-occ-18479-first-national-bank; us-occ-17710-first-national-bank; us-occ-18787-first-national-bank; us-occ-14252-first-national-bank; us-occ-8205-first-national-bank; us-occ-18125-first-national-bank; us-occ-7647-first-national-bank; us-occ-13742-first-national-bank; us-occ-14146-first-national-bank; us-occ-13170-first-national-bank</t>
+          <t>us-occ-18479-first-national-bank; NK-VEUcR2WqX6PU6EAJe9248K; NK-PQKV6m5qiHTwLDWU7iXqBn; us-occ-17324-first-national-bank; us-occ-21610-first-national-bank; us-occ-3496-first-national-bank; NK-aHpDcBPsCBsGiDs3VB9FMV; us-occ-11968-first-national-bank; NK-RPrxx7QDMC48WoRtfsVSYZ; us-occ-17710-first-national-bank; us-occ-18787-first-national-bank; us-occ-14163-first-national-bank; us-occ-8205-first-national-bank; NK-hNd7gSkdsgEtc2Cu2ehWpY; us-occ-13742-first-national-bank; us-occ-10230-first-national-bank; us-occ-7853-first-national-bank; us-occ-14252-first-national-bank; us-occ-12423-first-national-bank; us-occ-13830-first-national-bank; us-occ-14146-first-national-bank; us-occ-14012-first-national-bank; us-occ-20214-first-national-bank; us-occ-18125-first-national-bank; us-occ-17129-first-national-bank; us-occ-13170-first-national-bank; us-occ-7647-first-national-bank</t>
         </is>
       </c>
       <c r="H120" t="inlineStr"/>
@@ -5154,7 +5162,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>us-bis-export-173fea845bf18b35427a8c7824154f304ae92699; us-bis-export-4e4521de256e257e56ef540cfc9615fbca58ffd5; us-bis-export-3b4d4492559520a3a05364d87c5eb1ece6a3d45a; us-bis-export-a295516ab84e22c1ca78728dbf583db0ada3a5ee; us-bis-export-e25dae8aa140bb74e933673805dd812947f804f9; us-bis-export-06b4ca1f7407964e2eba031e7e7c71ce709bf5cb; us-bis-export-a61e141b1d62ffa7e7a023963c919bc16973ad6a; us-bis-export-85dd67671800490ba3681fb8ad28d2e8b105b77f; us-bis-export-2d2c0e1138134465184f8329dd9a9e2bd488eaea; us-bis-export-3c6e2c91f157b087fa544e2497b6a8a90f907b41; us-bis-export-218a8dc6b04ba337c56129a9b165ebfe49a27a24; us-bis-export-dc14fce64c4e0344ef0aaf83892b632b61068731; us-bis-export-8776a0f9f9a1b5d1b562f062afa4a3d92b28a4ac; us-bis-export-bf74de0594ae191f4f89580009eecd148fcf50c0; us-bis-export-17ad59fc4ad80c3eca72d9d1960843b8a8705b61; us-bis-export-bb54c8f154f6d8ce4de98322c2dfbddf266fb061; us-bis-export-281fab4da84b7335092ecd16a3ce755c7f9eaae7; us-bis-export-3d1c12f3588b6b7bc5465a3ab8fa5b1881450ccf; us-bis-export-0a6a060300638f2e79b43e087850dc51f22817b5; us-bis-export-1404eb90b660ca2d82253d519bfae2c4b99c6d43; us-bis-export-a72b992940743df5f0a6f4ccb0f1e08291cf1778; us-bis-export-31b7a14650406324db7fb583916ff654aa71ad0d; us-bis-export-afb52eaf128f3585a1175a56f1a28ec428feda70; us-bis-export-5edd5ab23cf265aa0a67b045caa2f8eadf834601; us-bis-export-9e4ddd0e1750640de0b220a6e2d0dadf485ce945; us-bis-export-45f6f4d88223f01f73d042e6d82e278da68f3c2a; us-bis-export-fedf7749dac3e962046a9dd7f2a16eb1664d1564</t>
+          <t>us-bis-export-a61e141b1d62ffa7e7a023963c919bc16973ad6a; us-bis-export-4e4521de256e257e56ef540cfc9615fbca58ffd5; us-bis-export-afb52eaf128f3585a1175a56f1a28ec428feda70; us-bis-export-bf74de0594ae191f4f89580009eecd148fcf50c0; us-bis-export-3d1c12f3588b6b7bc5465a3ab8fa5b1881450ccf; us-bis-export-2d2c0e1138134465184f8329dd9a9e2bd488eaea; us-bis-export-5edd5ab23cf265aa0a67b045caa2f8eadf834601; us-bis-export-fedf7749dac3e962046a9dd7f2a16eb1664d1564; us-bis-export-31b7a14650406324db7fb583916ff654aa71ad0d; us-bis-export-06b4ca1f7407964e2eba031e7e7c71ce709bf5cb; us-bis-export-0a6a060300638f2e79b43e087850dc51f22817b5; us-bis-export-3b4d4492559520a3a05364d87c5eb1ece6a3d45a; us-bis-export-17ad59fc4ad80c3eca72d9d1960843b8a8705b61; us-bis-export-bb54c8f154f6d8ce4de98322c2dfbddf266fb061; us-bis-export-e25dae8aa140bb74e933673805dd812947f804f9; us-bis-export-85dd67671800490ba3681fb8ad28d2e8b105b77f; us-bis-export-1404eb90b660ca2d82253d519bfae2c4b99c6d43; us-bis-export-a295516ab84e22c1ca78728dbf583db0ada3a5ee; us-bis-export-45f6f4d88223f01f73d042e6d82e278da68f3c2a; us-bis-export-8776a0f9f9a1b5d1b562f062afa4a3d92b28a4ac; us-bis-export-281fab4da84b7335092ecd16a3ce755c7f9eaae7; us-bis-export-a72b992940743df5f0a6f4ccb0f1e08291cf1778; us-bis-export-dc14fce64c4e0344ef0aaf83892b632b61068731; us-bis-export-218a8dc6b04ba337c56129a9b165ebfe49a27a24; us-bis-export-9e4ddd0e1750640de0b220a6e2d0dadf485ce945; us-bis-export-173fea845bf18b35427a8c7824154f304ae92699; us-bis-export-3c6e2c91f157b087fa544e2497b6a8a90f907b41</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -5193,7 +5201,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>isin-RU000A105SX7; isin-RU000A106JZ9; isin-RU000A1078H1; isin-RU000A106K27; isin-RU000A107217; isin-RU000A107KV4; isin-RU000A107456; isin-RU000A105CM4; isin-RU000A106UW3; isin-RU000A106SE5; isin-RU000A107AG6; isin-RU000A104W58; isin-RU000A101XH9; isin-RU000A105AW7; isin-RU000A1030X9; isin-RU000A102VW0; isin-RU000A104ZV9; isin-RU000A103KJ8; isin-RU000A103UY6; isin-RU000A106656; isin-RU000A104JB5; isin-RU000A105M91; isin-RU000A105M75; isin-RU000A105492; isin-RU000A103FP5; isin-RU000A101YD6</t>
+          <t>isin-RU000A103FP5; isin-RU000A105M75; isin-RU000A101XH9; isin-RU000A107AG6; isin-RU000A107456; isin-RU000A105M91; isin-RU000A1078H1; isin-RU000A1030X9; isin-RU000A104ZV9; isin-RU000A102VW0; isin-RU000A106K27; isin-RU000A105CM4; isin-RU000A104JB5; isin-RU000A105AW7; isin-RU000A106SE5; isin-RU000A105SX7; isin-RU000A101YD6; isin-RU000A107KV4; isin-RU000A106JZ9; isin-RU000A104W58; isin-RU000A107217; isin-RU000A105492; isin-RU000A106656; isin-RU000A106UW3; isin-RU000A103UY6; isin-RU000A103KJ8</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -5232,7 +5240,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>isin-RU000A103BQ2; isin-RU000A10D533; isin-RU000A103BR0; isin-RU000A1038Z7; isin-RU000A10D517; isin-RU000A108EG6; isin-RU000A102BT8; isin-RU000A1074G2; isin-RU000A101QE0; isin-RU000A1038V6; isin-RU000A10BVC8; isin-RU000A108EE1; isin-RU000A106E90; isin-RU000A105RV3; isin-RU000A10CKT3; isin-RU000A108EH4; isin-RU000A105FZ9; isin-RU000A108EF8; isin-RU000A10D4Y2; isin-RU000A1028E3; isin-RU000A101F94; isin-RU000A1014N4; isin-RU000A10BVH7; isin-RU000A101FA1; isin-RU000A103901</t>
+          <t>isin-RU000A1038V6; isin-RU000A101F94; isin-RU000A1014N4; isin-RU000A108EF8; isin-RU000A10BVH7; isin-RU000A10D517; isin-RU000A101FA1; isin-RU000A108EG6; isin-RU000A105RV3; isin-RU000A103901; isin-RU000A101QE0; isin-RU000A102BT8; isin-RU000A103BQ2; isin-RU000A108EH4; isin-RU000A105FZ9; isin-RU000A108EE1; isin-RU000A106E90; isin-RU000A10CKT3; isin-RU000A1074G2; isin-RU000A10BVC8; isin-RU000A1028E3; isin-RU000A103BR0; isin-RU000A10D533; isin-RU000A1038Z7; isin-RU000A10D4Y2</t>
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
@@ -5271,7 +5279,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>isin-RU000A107QM0; isin-RU000A10BV55; isin-RU000A10DPT0; isin-RU000A107U65; isin-RU000A10B3A6; isin-RU000A10DEE6; isin-RU000A10DSU2; isin-RU000A10ASQ6; isin-RU000A10B008; isin-RU000A10CCJ1; isin-RU000A1082Y8; isin-RU000A10B4U2; isin-RU000A10EG28; isin-RU000A10A6W4; isin-RU000A10BS76; isin-RU000A10C741; isin-RU000A10CZ35; isin-RU000A10CZ43; isin-RU000A10B396; isin-RU000A106QS9; isin-RU000A107ST1; isin-RU000A10C5L7; isin-RU000A108AK6; isin-RU000A10AXP8; isin-RU000A10C5J1</t>
+          <t>isin-RU000A1082Y8; isin-RU000A10B396; isin-RU000A10C741; isin-RU000A10B3A6; isin-RU000A10B4U2; isin-RU000A10BV55; isin-RU000A108AK6; isin-RU000A10C5J1; isin-RU000A10CZ35; isin-RU000A10DSU2; isin-RU000A107ST1; isin-RU000A106QS9; isin-RU000A10B008; isin-RU000A10DEE6; isin-RU000A10CCJ1; isin-RU000A10AXP8; isin-RU000A10CZ43; isin-RU000A10DPT0; isin-RU000A10C5L7; isin-RU000A10A6W4; isin-RU000A10BS76; isin-RU000A10ASQ6; isin-RU000A10EG28; isin-RU000A107U65; isin-RU000A107QM0</t>
         </is>
       </c>
       <c r="H124" t="inlineStr"/>
@@ -5310,7 +5318,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>isin-RU000A109HX2; isin-RU000A10B933; isin-RU000A10E7K3; isin-RU000A10AZF4; isin-RU000A107WD7; isin-RU000A10C8M9; isin-RU000A10EKZ6; isin-RU000A10B3T6; isin-RU000A10CRP6; isin-RU000A10BTQ2; isin-RU000A10DB16; isin-RU000A109LC8; isin-RU000A10B0S4; isin-RU000A10AXW4; isin-RU000A107QL2; isin-RU000A10BXV4; isin-RU000A10AUX8; isin-RU000A10ARS4; isin-RU000A1080Y2; isin-RU000A10BJ02; isin-RU000A109VK0; isin-RU000A107SH6; isin-RU000A109UD7; isin-RU000A107S85; isin-RU000A10BWC6</t>
+          <t>isin-RU000A10AUX8; isin-RU000A10C8M9; isin-RU000A10EKZ6; isin-RU000A10E7K3; isin-RU000A107S85; isin-RU000A109LC8; isin-RU000A107QL2; isin-RU000A109UD7; isin-RU000A10B933; isin-RU000A107WD7; isin-RU000A1080Y2; isin-RU000A10B0S4; isin-RU000A10B3T6; isin-RU000A10BTQ2; isin-RU000A10ARS4; isin-RU000A109HX2; isin-RU000A10BWC6; isin-RU000A10AZF4; isin-RU000A10AXW4; isin-RU000A10BJ02; isin-RU000A107SH6; isin-RU000A10DB16; isin-RU000A10CRP6; isin-RU000A10BXV4; isin-RU000A109VK0</t>
         </is>
       </c>
       <c r="H125" t="inlineStr"/>
@@ -5349,7 +5357,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>no-nbim-46ac91a077b6c024128c2c2b2f0f03f37db76c42; no-nbim-7825269fe6f067176238eb2339e7206ffcc151e8; no-nbim-a4d6faf199e47ddaa804fe8a6d9f0a8c8c71e58a; no-nbim-b85fe1c47acee66b1e7dd5f1a9df6dc26bea3b85; no-nbim-20325ad3083d0ff8ad422af46d970bc66fd2df4a; no-nbim-54a19ec5707a9151128df444880be1ee95ba4aa7; no-nbim-6842761b1f94e36a84558e70e02d51bbc026b7c8; no-nbim-43b691c38cd2ba339a26370b3960886320701a8f; no-nbim-54168605e905203ee16aa68cba04b6feba01f66e; no-nbim-14d5b73c7448e6d23a8af79484167db48f96cabb; no-nbim-d406f451b7171f33a4496dc638b1495fcf54ba65; no-nbim-7b5a5352f3a4d0bd7ebc83af08d513b439e3fbe9; no-nbim-2f7771e2b01547c1ed051a0f29af54fa0c96233e; no-nbim-dd4670872c7a1bc4a436d29402707fcd63b990ab; no-nbim-0c136825e3af083f0041685169e4a57c3e3466a7; no-nbim-80cf25833ca330c5a9011cd13aaac889ce7e3769; no-nbim-86df20911ff88d155973ba77ca148a0bf531cc22; no-nbim-4a220402953f34cd56e50670864f1de02710d28e; no-nbim-1977f3a41fc08cbc33794ef56f2e91e8943f6f84; no-nbim-0ee27d2d2189180162392c67cb1ecc5b711bc804; no-nbim-04113b29457e7dd9a46c0166be5f17ea12e448ea; no-nbim-4252715357037c18d58d2ec275d620657ec6cc8e; no-nbim-1e79f156fa7cbe04326ed3df5d7f137bc9b57964; no-nbim-f2bb9fef70fcf9962dce52d7cda87123a39fedcb; no-nbim-37d6a36229c9644daa288e26ac0923c46003e01d</t>
+          <t>no-nbim-d406f451b7171f33a4496dc638b1495fcf54ba65; no-nbim-04113b29457e7dd9a46c0166be5f17ea12e448ea; no-nbim-43b691c38cd2ba339a26370b3960886320701a8f; no-nbim-0ee27d2d2189180162392c67cb1ecc5b711bc804; no-nbim-80cf25833ca330c5a9011cd13aaac889ce7e3769; no-nbim-37d6a36229c9644daa288e26ac0923c46003e01d; no-nbim-6842761b1f94e36a84558e70e02d51bbc026b7c8; no-nbim-1e79f156fa7cbe04326ed3df5d7f137bc9b57964; no-nbim-1977f3a41fc08cbc33794ef56f2e91e8943f6f84; no-nbim-7825269fe6f067176238eb2339e7206ffcc151e8; no-nbim-20325ad3083d0ff8ad422af46d970bc66fd2df4a; no-nbim-7b5a5352f3a4d0bd7ebc83af08d513b439e3fbe9; no-nbim-a4d6faf199e47ddaa804fe8a6d9f0a8c8c71e58a; no-nbim-0c136825e3af083f0041685169e4a57c3e3466a7; no-nbim-2f7771e2b01547c1ed051a0f29af54fa0c96233e; no-nbim-54168605e905203ee16aa68cba04b6feba01f66e; no-nbim-54a19ec5707a9151128df444880be1ee95ba4aa7; no-nbim-dd4670872c7a1bc4a436d29402707fcd63b990ab; no-nbim-86df20911ff88d155973ba77ca148a0bf531cc22; no-nbim-4a220402953f34cd56e50670864f1de02710d28e; no-nbim-46ac91a077b6c024128c2c2b2f0f03f37db76c42; no-nbim-4252715357037c18d58d2ec275d620657ec6cc8e; no-nbim-b85fe1c47acee66b1e7dd5f1a9df6dc26bea3b85; no-nbim-14d5b73c7448e6d23a8af79484167db48f96cabb; no-nbim-f2bb9fef70fcf9962dce52d7cda87123a39fedcb</t>
         </is>
       </c>
       <c r="H126" t="inlineStr"/>
@@ -5388,7 +5396,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>isin-RU000A10C6M3; isin-RU000A10DYB0; isin-RU000A1099W6; isin-RU000A10DE54; isin-RU000A10AC67; isin-RU000A10E291; isin-RU000A10EG44; isin-RU000A109SJ8; isin-RU000A10DCE0; isin-RU000A107R29; isin-RU000A10B2P6; isin-RU000A10D4W6; isin-RU000A10ED62; isin-RU000A10CH03; isin-RU000A10AHB1; isin-RU000A10BQX4; isin-RU000A10E7U2; isin-RU000A10BHY1; isin-RU000A10DY84; isin-RU000A10EMT5; isin-RU000A10A398; isin-RU000A10BTT6; isin-RU000A107SG8; isin-RU000A1099E4</t>
+          <t>isin-RU000A10BHY1; isin-RU000A107SG8; isin-RU000A10EG44; isin-RU000A10BTT6; isin-RU000A10CH03; isin-RU000A1099E4; isin-RU000A10AHB1; isin-RU000A107R29; isin-RU000A10A398; isin-RU000A10AC67; isin-RU000A10E7U2; isin-RU000A109SJ8; isin-RU000A10DYB0; isin-RU000A10EMT5; isin-RU000A10E291; isin-RU000A10B2P6; isin-RU000A10BQX4; isin-RU000A10DE54; isin-RU000A10ED62; isin-RU000A10D4W6; isin-RU000A10C6M3; isin-RU000A10DY84; isin-RU000A10DCE0; isin-RU000A1099W6</t>
         </is>
       </c>
       <c r="H127" t="inlineStr"/>
@@ -5427,7 +5435,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>sg-gov-a93e63023e86ca5386b8bb23dd755c74bbc95e50; sg-gov-2580ce11f24ca1d0d4874fc5969477fb433fec20; sg-gov-5e39ca8dd413db5428515dc7a00494bdd4da858e; sg-gov-d1a6df395955e8a6877de5a6cda9bc290e46101d; sg-gov-c829f977424d64b7986e37d0be7a7b6e3ad0523e; sg-gov-cf2dd9d128ecec72bf3b44af1dce9953666281d1; sg-gov-fd12b676f4351cdfc9dc60d1e79e93415a4eb3dc; sg-gov-94fc488595eb577cd6ba2705b92c3482b4e02425; sg-gov-d1bca9c114e1a89a6512eb125e6c59a40672f237; sg-gov-9814022a95cd6bc0beea8501d4e10f03738a84dc; sg-gov-2fc6f733cd9085bef8aee4dde734b49e392b4c85; sg-gov-614c74afa47eced172ed3f668fff503e229ce552; sg-gov-62f44c94332d3be8bc8cff76681436955dec35f4; sg-gov-9a96fd0bf768a09822c966b7b44eb5e76a6934b9; sg-gov-ae9e3a5efb2b35f3205437449cd0adfd719c8bf9; sg-gov-013e1d8d8032a9c7bc6036919935f2b093af042b; sg-gov-3301993066bbd63cd5afc2e1d176a34c5d36dfcd; sg-gov-64fa8dfbe7b96401b8b33a848c18220bb9b9e9e6; sg-gov-1927ac2500e15defba3f881a7bb6a848c4d567dd; sg-gov-db6ee8c9d9074ae4e4e5e785f197b92c2ebc147b; sg-gov-4d6ca2a0fc046c0616ff2b69bd0c0c9c4485b16e; sg-gov-0019b5723ae2b3bab694a56a064525cb3e070196; sg-gov-828fcb00f515ba3853dd3753b352841cafead58d; sg-gov-794729f23280383e04b16a261c769042e33ed6a9</t>
+          <t>sg-gov-794729f23280383e04b16a261c769042e33ed6a9; sg-gov-9a96fd0bf768a09822c966b7b44eb5e76a6934b9; sg-gov-614c74afa47eced172ed3f668fff503e229ce552; sg-gov-2fc6f733cd9085bef8aee4dde734b49e392b4c85; sg-gov-3301993066bbd63cd5afc2e1d176a34c5d36dfcd; sg-gov-828fcb00f515ba3853dd3753b352841cafead58d; sg-gov-c829f977424d64b7986e37d0be7a7b6e3ad0523e; sg-gov-4d6ca2a0fc046c0616ff2b69bd0c0c9c4485b16e; sg-gov-5e39ca8dd413db5428515dc7a00494bdd4da858e; sg-gov-d1a6df395955e8a6877de5a6cda9bc290e46101d; sg-gov-1927ac2500e15defba3f881a7bb6a848c4d567dd; sg-gov-a93e63023e86ca5386b8bb23dd755c74bbc95e50; sg-gov-62f44c94332d3be8bc8cff76681436955dec35f4; sg-gov-94fc488595eb577cd6ba2705b92c3482b4e02425; sg-gov-013e1d8d8032a9c7bc6036919935f2b093af042b; sg-gov-d1bca9c114e1a89a6512eb125e6c59a40672f237; sg-gov-ae9e3a5efb2b35f3205437449cd0adfd719c8bf9; sg-gov-2580ce11f24ca1d0d4874fc5969477fb433fec20; sg-gov-64fa8dfbe7b96401b8b33a848c18220bb9b9e9e6; sg-gov-db6ee8c9d9074ae4e4e5e785f197b92c2ebc147b; sg-gov-0019b5723ae2b3bab694a56a064525cb3e070196; sg-gov-9814022a95cd6bc0beea8501d4e10f03738a84dc; sg-gov-fd12b676f4351cdfc9dc60d1e79e93415a4eb3dc; sg-gov-cf2dd9d128ecec72bf3b44af1dce9953666281d1</t>
         </is>
       </c>
       <c r="H128" t="inlineStr"/>
@@ -5466,7 +5474,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>isin-RU000A102B48; isin-RU000A106P63; isin-RU000A1043Z7; isin-RU000A107001; isin-RU000A1022G1; isin-RU000A105WC3; isin-RU000A102200; isin-RU000A107GV2; isin-RU000A106HF5; isin-RU000A102KU7; isin-RU000A102AK9; isin-RU000A1060Q0; isin-RU000A105XF4; isin-RU000A103CD8; isin-RU000A105Q89; isin-RU000A106U90; isin-RU000A106UM4; isin-RU000A1074Q1; isin-RU000A102J57; isin-RU000A102T97; isin-RU000A103QK3; isin-RU000A1060X6</t>
+          <t>isin-RU000A105WC3; isin-RU000A102J57; isin-RU000A1022G1; isin-RU000A102200; isin-RU000A107GV2; isin-RU000A1060Q0; isin-RU000A105Q89; isin-RU000A102AK9; isin-RU000A103CD8; isin-RU000A103QK3; isin-RU000A106UM4; isin-RU000A106HF5; isin-RU000A1074Q1; isin-RU000A102B48; isin-RU000A102T97; isin-RU000A1060X6; isin-RU000A106P63; isin-RU000A102KU7; isin-RU000A105XF4; isin-RU000A106U90; isin-RU000A1043Z7; isin-RU000A107001</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -5505,7 +5513,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>isin-RU000A10B6K8; isin-RU000A108FS8; isin-RU000A10BRY0; isin-RU000A10CST6; isin-RU000A10EFW3; isin-RU000A10DLY9; isin-RU000A10B5M6; isin-RU000A10DTU0; isin-RU000A10B7S9; isin-RU000A10E9M5; isin-RU000A10CJ84; isin-RU000A109R50; isin-RU000A109QQ7; isin-RU000A10B5A1; isin-RU000A10E5Y8; isin-RU000A10DD97; isin-RU000A10ADD6; isin-RU000A108E80; isin-RU000A10A1N4; isin-RU000A1094W7; isin-RU000A10DA58; isin-RU000A107W71</t>
+          <t>isin-RU000A109R50; isin-RU000A10B7S9; isin-RU000A108E80; isin-RU000A10CST6; isin-RU000A10B6K8; isin-RU000A109QQ7; isin-RU000A108FS8; isin-RU000A10A1N4; isin-RU000A10BRY0; isin-RU000A1094W7; isin-RU000A10DA58; isin-RU000A10E9M5; isin-RU000A10E5Y8; isin-RU000A10B5A1; isin-RU000A10DTU0; isin-RU000A107W71; isin-RU000A10EFW3; isin-RU000A10ADD6; isin-RU000A10DD97; isin-RU000A10B5M6; isin-RU000A10DLY9; isin-RU000A10CJ84</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -5544,7 +5552,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>us-bis-export-95e00cf9524edf302d6a5d8ada933810c3ef58bd; us-bis-export-e0f6ec8632de4d5956e691705e14e11f9e966621; us-bis-export-31b5980d59cad15f717ea5a0f834828197a31378; us-bis-export-b6d9a86e73c8a14cc3f69098c077f0a477bd50ff; us-bis-export-a78c7b4be367a59af55ba73a79de0e3ea863be11; us-bis-export-5c42d11d5978ac49d3245471a4391a7a7f887cec; us-bis-export-8ab589564d10f1a1bfc884342d729d801365f078; us-bis-export-b194b89e3edad175738bbf00c0a5d0aa04c32c7e; us-bis-export-d9c3f96987659b69729b05579ce9cb6f01d311ef; us-bis-export-f1871aecb94cc579532c623408bbd19d88d76a81; us-bis-export-070a9418024dc4c861eaaaa578715d281c579d20; us-bis-export-dc7b2e7354e58f567d74c8b82986427353a7217a; us-bis-export-0bd4567190959cfc6a293f3406a6535040771c63; us-bis-export-99ce99a9d90710c2dac70c609aaeaea3943465c3; us-bis-export-20bb29356a300e96fe7450126f4ddf9bd8af9eb4; us-bis-export-7b75563abace54b3750b066822080b27054e006b; us-bis-export-e9284d5d6ae34f203de5ae376a0e8aaa8b6b6d01; us-bis-export-0bcd76f3bae9b241d3fcb3af2ff43fab510e891c; us-bis-export-ca81a679e19a211e7cfc19a8741fcdc6ab3f2bd8; us-bis-export-67e260a57a8b4765a8569cf0b4dff53040d04aa1; us-bis-export-bba74fdbbd08546826f71684bf523e17390b704c; us-bis-export-aa6ac67a6e6a0368faf3a4af1ae3926a5a160f48</t>
+          <t>us-bis-export-20bb29356a300e96fe7450126f4ddf9bd8af9eb4; us-bis-export-e0f6ec8632de4d5956e691705e14e11f9e966621; us-bis-export-b6d9a86e73c8a14cc3f69098c077f0a477bd50ff; us-bis-export-e9284d5d6ae34f203de5ae376a0e8aaa8b6b6d01; us-bis-export-ca81a679e19a211e7cfc19a8741fcdc6ab3f2bd8; us-bis-export-070a9418024dc4c861eaaaa578715d281c579d20; us-bis-export-95e00cf9524edf302d6a5d8ada933810c3ef58bd; us-bis-export-f1871aecb94cc579532c623408bbd19d88d76a81; us-bis-export-bba74fdbbd08546826f71684bf523e17390b704c; us-bis-export-0bd4567190959cfc6a293f3406a6535040771c63; us-bis-export-aa6ac67a6e6a0368faf3a4af1ae3926a5a160f48; us-bis-export-99ce99a9d90710c2dac70c609aaeaea3943465c3; us-bis-export-a78c7b4be367a59af55ba73a79de0e3ea863be11; us-bis-export-7b75563abace54b3750b066822080b27054e006b; us-bis-export-b194b89e3edad175738bbf00c0a5d0aa04c32c7e; us-bis-export-5c42d11d5978ac49d3245471a4391a7a7f887cec; us-bis-export-67e260a57a8b4765a8569cf0b4dff53040d04aa1; us-bis-export-31b5980d59cad15f717ea5a0f834828197a31378; us-bis-export-d9c3f96987659b69729b05579ce9cb6f01d311ef; us-bis-export-0bcd76f3bae9b241d3fcb3af2ff43fab510e891c; us-bis-export-dc7b2e7354e58f567d74c8b82986427353a7217a; us-bis-export-8ab589564d10f1a1bfc884342d729d801365f078</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -5583,7 +5591,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>us-bis-export-cd23502eefc825a42b55ff0a4706a3e732059477; us-bis-export-bc925a30a4c841245755ea1080e11db9f5778918; us-bis-export-2f4847eb6d7000565f5634ab49dbcb2529d7e52a; us-bis-export-838f40aae3d8c2c6b820d53373786da022bbad31; us-bis-export-5c319d600981b5db3266bc71c1bbfb5138847a59; us-bis-export-e61e6d2c7005b45d4aa26a0bf6838cdc2e1e0d06; us-bis-export-71bbfa7d8e06753f33eb55750f90f0b83900e650; us-bis-export-0f4075cdfaef34bc63acdebb7f28a331d4ba55e7; us-bis-export-fae583b4d3b4960813de4e9898954dccc65307c1; us-bis-export-751a34d9931eda6d59b0b01ebad576a04fe69c21; us-bis-export-2835c8b6ce5e23de2b1089574f821c2e8c35d636; us-bis-export-eb93fd0e4e8300d577ae1d93ede9a4648b5b2e4f; us-bis-export-20809edf4fb94a271cfe4a46bfb2fe8289f1ff24; us-bis-export-69d87f6441baaee676e8805be4a9c33a108e80cb; us-bis-export-a66c36ad213a6d3de23572c73c046d1f815365c2; us-bis-export-8f1d8eb816688c0121d436c54c8052c4adc31134; us-bis-export-ca6e412b1391ca54f63947807d98479d1a671f76; us-bis-export-5011cf717c40b95c8c47561cee6035c9bf703ea8; us-bis-export-460a88d54d1e453481b038cb41a8733fdb2f2748; us-bis-export-bdbfcd189c60bb175c4239da0b539a4089b02c9d; us-bis-export-bfc72336fb63d1f44bab067cf035e93ede5f9678; us-bis-export-c612f655270fc0f7a1943e189575bc7c13cb171e</t>
+          <t>us-bis-export-71bbfa7d8e06753f33eb55750f90f0b83900e650; us-bis-export-e61e6d2c7005b45d4aa26a0bf6838cdc2e1e0d06; us-bis-export-bc925a30a4c841245755ea1080e11db9f5778918; us-bis-export-69d87f6441baaee676e8805be4a9c33a108e80cb; us-bis-export-5011cf717c40b95c8c47561cee6035c9bf703ea8; us-bis-export-eb93fd0e4e8300d577ae1d93ede9a4648b5b2e4f; us-bis-export-fae583b4d3b4960813de4e9898954dccc65307c1; us-bis-export-751a34d9931eda6d59b0b01ebad576a04fe69c21; us-bis-export-8f1d8eb816688c0121d436c54c8052c4adc31134; us-bis-export-ca6e412b1391ca54f63947807d98479d1a671f76; us-bis-export-a66c36ad213a6d3de23572c73c046d1f815365c2; us-bis-export-bfc72336fb63d1f44bab067cf035e93ede5f9678; us-bis-export-c612f655270fc0f7a1943e189575bc7c13cb171e; us-bis-export-0f4075cdfaef34bc63acdebb7f28a331d4ba55e7; us-bis-export-460a88d54d1e453481b038cb41a8733fdb2f2748; us-bis-export-2835c8b6ce5e23de2b1089574f821c2e8c35d636; us-bis-export-cd23502eefc825a42b55ff0a4706a3e732059477; us-bis-export-2f4847eb6d7000565f5634ab49dbcb2529d7e52a; us-bis-export-838f40aae3d8c2c6b820d53373786da022bbad31; us-bis-export-5c319d600981b5db3266bc71c1bbfb5138847a59; us-bis-export-bdbfcd189c60bb175c4239da0b539a4089b02c9d; us-bis-export-20809edf4fb94a271cfe4a46bfb2fe8289f1ff24</t>
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
@@ -5622,7 +5630,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>us-bis-export-4bf84b55868526c30a4c95b516454f1b611be1a1; us-bis-export-d84f17b0e98705fcfcd6c07897d4add05a1f4404; us-bis-export-e10f750a97f3e46190458feca8d78a9130ffca0c; us-bis-export-bbdc1db8da8709558874164e7b0a5e77fbf670d2; us-bis-export-99df182ea8c36e108d01be191737ae533c11bbcf; us-bis-export-a700af94468f7e84c736555b50e17764dbde29d3; us-bis-export-d82dc72cb2cf2776e188f49912a409550a26d711; us-bis-export-b95635194a5c1d4439d6efb227dfa1889142b79a; us-bis-export-7cb9ddd92a5af29c594fb4805f8c6932988a2ed7; us-bis-export-9acc1f3076edd878c7e9489d31a88b8fc99e004f; us-bis-export-e359171f0ec9509c16f390dfab8be4664982edf2; us-bis-export-495d5ef999a879ccf323201668b97b43bd2bebb2; us-bis-export-261df25e91433e816c44515004bb5f958d7fd06c; us-bis-export-6a2e184f7f129f3af838dde84fc883f7c8ed728e; us-bis-export-61b7348ec1e9088dc6b738dba3bbf5123faa65f7; us-bis-export-d616b39ea7d079d489420297559be1ff62eded96; us-bis-export-209182617447ec396edbd9f87bca3183a40ea2c6; us-bis-export-7e1dc1faeb06317f0b0e7003d7264536facdfce7; us-bis-export-45547edf9716ca47f9f50f7d4cfdc0b0c7b6c331; us-bis-export-879c73573486390fa1393639d0277f7723f3abe4; us-bis-export-5bc48fc45185208bfeafad3af72be80a0eb4cb7f; us-bis-export-c3645c67ae58b75aef7f8fd4797aa4cfa2d38c35</t>
+          <t>us-bis-export-bbdc1db8da8709558874164e7b0a5e77fbf670d2; us-bis-export-61b7348ec1e9088dc6b738dba3bbf5123faa65f7; us-bis-export-b95635194a5c1d4439d6efb227dfa1889142b79a; us-bis-export-261df25e91433e816c44515004bb5f958d7fd06c; us-bis-export-a700af94468f7e84c736555b50e17764dbde29d3; us-bis-export-45547edf9716ca47f9f50f7d4cfdc0b0c7b6c331; us-bis-export-209182617447ec396edbd9f87bca3183a40ea2c6; us-bis-export-5bc48fc45185208bfeafad3af72be80a0eb4cb7f; us-bis-export-99df182ea8c36e108d01be191737ae533c11bbcf; us-bis-export-4bf84b55868526c30a4c95b516454f1b611be1a1; us-bis-export-7cb9ddd92a5af29c594fb4805f8c6932988a2ed7; us-bis-export-d84f17b0e98705fcfcd6c07897d4add05a1f4404; us-bis-export-495d5ef999a879ccf323201668b97b43bd2bebb2; us-bis-export-d616b39ea7d079d489420297559be1ff62eded96; us-bis-export-e359171f0ec9509c16f390dfab8be4664982edf2; us-bis-export-d82dc72cb2cf2776e188f49912a409550a26d711; us-bis-export-e10f750a97f3e46190458feca8d78a9130ffca0c; us-bis-export-879c73573486390fa1393639d0277f7723f3abe4; us-bis-export-c3645c67ae58b75aef7f8fd4797aa4cfa2d38c35; us-bis-export-7e1dc1faeb06317f0b0e7003d7264536facdfce7; us-bis-export-9acc1f3076edd878c7e9489d31a88b8fc99e004f; us-bis-export-6a2e184f7f129f3af838dde84fc883f7c8ed728e</t>
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
@@ -5661,7 +5669,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>isin-RU000A10D4P0; isin-RU000A10E6D0; isin-RU000A1097C2; isin-RU000A108GM9; isin-RU000A10B2X0; isin-RU000A107UB5; isin-RU000A10C9Y2; isin-RU000A10C5K9; isin-RU000A10A4C1; isin-RU000A1082K7; isin-RU000A10BFG2; isin-RU000A108WV7; isin-RU000A10B4W8; isin-RU000A10A6U8; isin-RU000A10BJ85; isin-RU000A10B3X8; isin-RU000A107U40; isin-RU000A10B750; isin-RU000A10AV31; isin-RU000A10BWL7; isin-RU000A107W06</t>
+          <t>isin-RU000A10BFG2; isin-RU000A10C5K9; isin-RU000A10C9Y2; isin-RU000A10AV31; isin-RU000A10D4P0; isin-RU000A10A4C1; isin-RU000A108WV7; isin-RU000A10B2X0; isin-RU000A10A6U8; isin-RU000A10B4W8; isin-RU000A107UB5; isin-RU000A107U40; isin-RU000A1097C2; isin-RU000A10BWL7; isin-RU000A1082K7; isin-RU000A107W06; isin-RU000A10B3X8; isin-RU000A10B750; isin-RU000A10BJ85; isin-RU000A10E6D0; isin-RU000A108GM9</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
@@ -5700,7 +5708,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>us-bis-export-8aaf946ddb3c987d32f2735fc1a3a1c58e4e7097; us-bis-export-a932b66db5e2cb883f8e9f62795682a3d2793c0e; us-bis-export-62895e8eac035752ce9c8b9f895aa0df96368b9a; us-bis-export-2d2e65a0f060212aee1ef47e581a7ac389202b8f; us-bis-export-539e60427aabf99c9c6c268d51e373b63f2e8a33; us-bis-export-74c75668144750df248c0934eeeda17cc295fa64; us-bis-export-49eee0e9a1d21bd7b32e94ea237ccae74717742e; us-bis-export-020d0ffa4f3afcce77f012d727b467d317e7e9db; us-bis-export-4f15715bfa15bb1d1bbbef4f26261b414354858e; us-bis-export-35ca9b34585a509b4da8a62069c5961dc9bcc934; us-bis-export-1fe7b1caf8fef630e7d824dc2b04745e6dd6256d; us-bis-export-f3381c93f958c84e2ccb561654155a8cfeebde71; us-bis-export-83b2b506e661eab620190113dbdb874c38992aef; us-bis-export-d75a538d6160f8834824bbc8d7ca626d60de657e; us-bis-export-e73bb9f346a85cba47fe1377ca0c12e881572cdb; us-bis-export-5944af2a6b2433236a79fa36d0f03dac37c06035; us-bis-export-2603358c5b2f6847657a8972e20a62b24fe638c4; us-bis-export-43caa771a65771f1fbb3c487692074dd99eae30d; us-bis-export-8b43476bc109335dcf2be663a2e6996e22762136; us-bis-export-3ac4d5f3a4cf9c2c5f75fecd80455e5cfcce7492; us-bis-export-66cea3a7fe3da5a638361f251fbd1a5e92b7d560</t>
+          <t>us-bis-export-539e60427aabf99c9c6c268d51e373b63f2e8a33; us-bis-export-a932b66db5e2cb883f8e9f62795682a3d2793c0e; us-bis-export-35ca9b34585a509b4da8a62069c5961dc9bcc934; us-bis-export-8aaf946ddb3c987d32f2735fc1a3a1c58e4e7097; us-bis-export-e73bb9f346a85cba47fe1377ca0c12e881572cdb; us-bis-export-3ac4d5f3a4cf9c2c5f75fecd80455e5cfcce7492; us-bis-export-2d2e65a0f060212aee1ef47e581a7ac389202b8f; us-bis-export-74c75668144750df248c0934eeeda17cc295fa64; us-bis-export-5944af2a6b2433236a79fa36d0f03dac37c06035; us-bis-export-43caa771a65771f1fbb3c487692074dd99eae30d; us-bis-export-2603358c5b2f6847657a8972e20a62b24fe638c4; us-bis-export-1fe7b1caf8fef630e7d824dc2b04745e6dd6256d; us-bis-export-49eee0e9a1d21bd7b32e94ea237ccae74717742e; us-bis-export-020d0ffa4f3afcce77f012d727b467d317e7e9db; us-bis-export-62895e8eac035752ce9c8b9f895aa0df96368b9a; us-bis-export-d75a538d6160f8834824bbc8d7ca626d60de657e; us-bis-export-66cea3a7fe3da5a638361f251fbd1a5e92b7d560; us-bis-export-4f15715bfa15bb1d1bbbef4f26261b414354858e; us-bis-export-83b2b506e661eab620190113dbdb874c38992aef; us-bis-export-8b43476bc109335dcf2be663a2e6996e22762136; us-bis-export-f3381c93f958c84e2ccb561654155a8cfeebde71</t>
         </is>
       </c>
       <c r="H135" t="inlineStr"/>
@@ -5739,7 +5747,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Q136745505; Q20500051; Q133539204; Q136979359; Q116056211; Q116056259; Q34526819; Q116056140; Q116055982; Q28603835; Q137794235; Q30723983; Q133820138; Q30755529; Q31192847; Q116056154; Q116056196; Q110070915; Q137595068</t>
+          <t>Q34526819; Q116056259; Q136745505; Q137595068; Q116055982; Q116056196; Q20500051; Q116056154; Q30755529; Q133539204; Q110070915; Q116056140; Q133820138; Q31192847; Q28603835; Q136979359; Q30723983; Q137794235; Q116056211</t>
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
@@ -5778,7 +5786,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>isin-RU000A1066D5; isin-RU000A102A49; isin-RU000A10D4Z9; isin-RU000A101N52; isin-RU000A10AA93; isin-RU000A101CK7; isin-RU000A105G16; isin-RU000A100QS2; isin-RU000A102BV4; isin-RU000A106Z61; isin-RU000A102A31; isin-RU000A1025A7; isin-RU000A1025B5; isin-RU000A10A7D2; isin-RU000A101KT1; isin-RU000A10D525; isin-RU000A105B11; isin-RU000A105L19; isin-RU000A1028D5</t>
+          <t>isin-RU000A100QS2; isin-RU000A1025A7; isin-RU000A1028D5; isin-RU000A10A7D2; isin-RU000A105B11; isin-RU000A101N52; isin-RU000A10AA93; isin-RU000A102BV4; isin-RU000A102A49; isin-RU000A105L19; isin-RU000A101CK7; isin-RU000A10D525; isin-RU000A102A31; isin-RU000A1025B5; isin-RU000A106Z61; isin-RU000A101KT1; isin-RU000A105G16; isin-RU000A1066D5; isin-RU000A10D4Z9</t>
         </is>
       </c>
       <c r="H137" t="inlineStr"/>
@@ -5817,7 +5825,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>isin-RU000A109817; isin-RU000A10EEL9; isin-RU000A10AZ03; isin-RU000A10C5X2; isin-RU000A107BJ8; isin-RU000A10BH38; isin-RU000A10BFU3; isin-RU000A10C2G4; isin-RU000A10EEU0; isin-RU000A10BH46; isin-RU000A106664; isin-RU000A109P60; isin-RU000A107UD1; isin-RU000A10B7Z4; isin-RU000A10BH04; isin-RU000A10DED8; isin-RU000A10DKT1; isin-RU000A108K41; isin-RU000A10BT91</t>
+          <t>isin-RU000A10AZ03; isin-RU000A10BH38; isin-RU000A10BT91; isin-RU000A10DED8; isin-RU000A10EEL9; isin-RU000A109817; isin-RU000A10C5X2; isin-RU000A106664; isin-RU000A10B7Z4; isin-RU000A10C2G4; isin-RU000A107UD1; isin-RU000A109P60; isin-RU000A10EEU0; isin-RU000A10BH46; isin-RU000A108K41; isin-RU000A107BJ8; isin-RU000A10BH04; isin-RU000A10BFU3; isin-RU000A10DKT1</t>
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
@@ -5856,7 +5864,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>isin-RU000A10D1C4; isin-RU000A10B5K0; isin-RU000A108QN6; isin-RU000A10CRR2; isin-RU000A108PJ6; isin-RU000A109X60; isin-RU000A10E5U6; isin-RU000A109F47; isin-RU000A10C2H2; isin-RU000A1099N5; isin-RU000A10A3E9; isin-RU000A10A6S2; isin-RU000A10E9T0; isin-RU000A109P94; isin-RU000A10AP13; isin-RU000A10C3C1; isin-RU000A10B7K6; isin-RU000A1099M7; isin-RU000A10AG89</t>
+          <t>isin-RU000A10E9T0; isin-RU000A10E5U6; isin-RU000A10C2H2; isin-RU000A109P94; isin-RU000A1099M7; isin-RU000A109F47; isin-RU000A108QN6; isin-RU000A10CRR2; isin-RU000A109X60; isin-RU000A10AP13; isin-RU000A10D1C4; isin-RU000A10A3E9; isin-RU000A1099N5; isin-RU000A10B7K6; isin-RU000A10B5K0; isin-RU000A108PJ6; isin-RU000A10AG89; isin-RU000A10A6S2; isin-RU000A10C3C1</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -5895,7 +5903,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>ru-b97bd09714e6b296aa6b71f11508ead3c927428f; ru-a94a261e1c395fd3f0b17b86415b4bece3d1fda7; ru-f841eecb6dcfede6347f7e198fac0191abd62d9b; ru-c196c159eede00171714dbd1e44ff7e8f121be86; ru-22b5dfc2c6f6845d5b336a501923b39963729da1; ru-90a64ab6f595aac0813340722527e78e7ad65e7f; ru-805da21ef189ec834359be7790272ba7891448bb; ru-9e9eaa6fa8fb5f871e8dcf20f84e4d5b1f5aaff4; ru-dbb1d6b680212b664c67ca872923a29b00ccf843; ru-67ca0d489769b18c0a473e21a1b64de3b19cd356; ru-e4d52d0d6e881b96b34c805407afd340b90e5286; ru-2255f7116450b3310dc43e58341e7c6cd9795472; ru-0b445022b0ec05fd6b34ae90e6f015a61ac43b32; ru-842769086a86a54eadd47780edad8d989983cb2e; ru-d33061f978495baf77808882721cda4dd668fb8f; ru-02f79694ce8503cd32cc193dd09de6b3bc4bf71c; ru-a3e8334bc3185ee1f3cda439c723355b9267abf3; ru-79738a69df052b67aa260d4c1980aaad822f1c3c; ru-1971ba12dbfff139a0eeaf75417a584b6e85d7e1</t>
+          <t>ru-805da21ef189ec834359be7790272ba7891448bb; ru-842769086a86a54eadd47780edad8d989983cb2e; ru-d33061f978495baf77808882721cda4dd668fb8f; ru-9e9eaa6fa8fb5f871e8dcf20f84e4d5b1f5aaff4; ru-67ca0d489769b18c0a473e21a1b64de3b19cd356; ru-b97bd09714e6b296aa6b71f11508ead3c927428f; ru-2255f7116450b3310dc43e58341e7c6cd9795472; ru-90a64ab6f595aac0813340722527e78e7ad65e7f; ru-a3e8334bc3185ee1f3cda439c723355b9267abf3; ru-22b5dfc2c6f6845d5b336a501923b39963729da1; ru-e4d52d0d6e881b96b34c805407afd340b90e5286; ru-0b445022b0ec05fd6b34ae90e6f015a61ac43b32; ru-02f79694ce8503cd32cc193dd09de6b3bc4bf71c; ru-a94a261e1c395fd3f0b17b86415b4bece3d1fda7; ru-f841eecb6dcfede6347f7e198fac0191abd62d9b; ru-79738a69df052b67aa260d4c1980aaad822f1c3c; ru-c196c159eede00171714dbd1e44ff7e8f121be86; ru-1971ba12dbfff139a0eeaf75417a584b6e85d7e1; ru-dbb1d6b680212b664c67ca872923a29b00ccf843</t>
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
@@ -5934,7 +5942,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>isin-RU000A102374; isin-RU000A101ZK8; isin-RU000A102Q90; isin-RU000A103D60; isin-RU000A101KR5; isin-RU000A102FD3; isin-RU000A102BC4; isin-RU000A101R74; isin-RU000A101UM5; isin-RU000A101MQ3; isin-RU000A103MY3; isin-RU000A102MW9; isin-RU000A102SL9; isin-RU000A1036C0; isin-RU000A103232; isin-RU000A102770; isin-RU000A103GZ2; isin-RU000A102YY0</t>
+          <t>isin-RU000A102YY0; isin-RU000A102SL9; isin-RU000A101ZK8; isin-RU000A102BC4; isin-RU000A102FD3; isin-RU000A103D60; isin-RU000A103MY3; isin-RU000A101UM5; isin-RU000A102MW9; isin-RU000A101KR5; isin-RU000A101R74; isin-RU000A102374; isin-RU000A101MQ3; isin-RU000A102770; isin-RU000A102Q90; isin-RU000A103232; isin-RU000A103GZ2; isin-RU000A1036C0</t>
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
@@ -5973,7 +5981,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>ru-inn-9714058147; ru-inn-5904037892; ru-inn-9728043461; ru-inn-7702527954; ru-inn-4101113738; ru-inn-7701657100; ru-inn-7704492383; ru-inn-9704194045; ru-inn-7725743542; ru-inn-6320085325; ru-inn-2531010480; ru-inn-7743289272; ru-inn-5507303700; ru-inn-7733711248; ru-inn-7701847158; ru-inn-5244022664; ru-inn-2308299972</t>
+          <t>ru-inn-5507303700; ru-inn-7702527954; ru-inn-9704194045; ru-inn-2308299972; ru-inn-4101113738; ru-inn-7743289272; ru-inn-9728043461; ru-inn-7701847158; ru-inn-7725743542; ru-inn-7733711248; ru-inn-6320085325; ru-inn-5244022664; ru-inn-5904037892; ru-inn-9714058147; ru-inn-7701657100; ru-inn-2531010480; ru-inn-7704492383</t>
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
@@ -6012,7 +6020,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>ua-edr-99df79a495063e953965645e3c0bb34f312f40a2; ua-edr-01627dafa2a14d4963b5d73f2a46624d71c97d7c; ua-edr-502c53beb1b493e2575fe161f8df265d6ce7eff4; ua-edr-429ddf533e5221aafb2d27580255bf6d189480c3; ua-edr-728dfe0fb5c472255c5d6676a3ee384785c5a62f; ua-edr-8bacf8ee166e0fc5abafd69917b524e0b3642103; ua-edr-9556f1bc706781002b4a1c78759637b93b530596; ua-edr-abc9cafe239f1758d1800119763500502ed6acd7; ua-edr-5e745987f6c7f714680d0b389c413b2df273ade3; ua-edr-841cbcb837a32baffda0de1e59414a89a6bee339; ua-edr-0877ee1e12f4cf3d331442fbb2ee500073e2f28c; ua-edr-f1f7d80410597a4639345afefd450f4feab86fbc; ua-edr-013090a414ba966e9b63fa324e4177ee0f20082b; ua-edr-a74c66ffe91a9489158df4ec8f91b0d647d4e8ce; ua-edr-ed93bcdb6a849d8ea9f0e733c2db19da3cf6eb52; ua-edr-5a986e1ed9b47d8b57f62a4189e7a87517ed3438; ua-edr-6002e691285c1f0f44c1bf301c1ac878cec8a859</t>
+          <t>ua-edr-a74c66ffe91a9489158df4ec8f91b0d647d4e8ce; ua-edr-f1f7d80410597a4639345afefd450f4feab86fbc; ua-edr-99df79a495063e953965645e3c0bb34f312f40a2; ua-edr-013090a414ba966e9b63fa324e4177ee0f20082b; ua-edr-ed93bcdb6a849d8ea9f0e733c2db19da3cf6eb52; ua-edr-429ddf533e5221aafb2d27580255bf6d189480c3; ua-edr-0877ee1e12f4cf3d331442fbb2ee500073e2f28c; ua-edr-5a986e1ed9b47d8b57f62a4189e7a87517ed3438; ua-edr-8bacf8ee166e0fc5abafd69917b524e0b3642103; ua-edr-502c53beb1b493e2575fe161f8df265d6ce7eff4; ua-edr-728dfe0fb5c472255c5d6676a3ee384785c5a62f; ua-edr-abc9cafe239f1758d1800119763500502ed6acd7; ua-edr-9556f1bc706781002b4a1c78759637b93b530596; ua-edr-01627dafa2a14d4963b5d73f2a46624d71c97d7c; ua-edr-6002e691285c1f0f44c1bf301c1ac878cec8a859; ua-edr-5e745987f6c7f714680d0b389c413b2df273ade3; ua-edr-841cbcb837a32baffda0de1e59414a89a6bee339</t>
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
@@ -6051,7 +6059,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>us-bis-export-9e57b0d8a1e9d2f89cc79b48ca81dc9ca509521d; us-bis-export-bb0c4774e8ff1b1b178c383784b9f07610e38caf; us-bis-export-535f1b58120e7716fa25ed80b1456b67c4156473; us-bis-export-ce7306e097264749e060f167284409070209a2c1; us-bis-export-f48912305c4dbcc6bb8632385fc391070974773d; us-bis-export-f59ed2b7aa0178d73365395b38ded03461840d95; us-bis-export-43bd1392fc4f3113c614c4c2b359c7adb2e31d79; us-bis-export-634ad637ca4a0ae524073c800a55e83a6ca5b091; us-bis-export-36fad77b3c3b0ed0ab420e0c78ba583f2c97eaec; us-bis-export-257a072ab7741aac127bbc27219b9e586a81fafd; us-bis-export-9642b172a01249feb8ddeda82ac3d0d8b7b2bb90; us-bis-export-03a3131d777c0b0575f941d28b30cfac7a0bfe61; us-bis-export-02a71f0a0b4df2ec61183537fd02e6a84266b4a4; us-bis-export-4dde4d81c422e0f99b9683ca4eb18c2392155e66; us-bis-export-41786fd0bd0a1322671f5091163b8bf2b12d149f; us-bis-export-995e9097a29d10642017db31ba22f09e344e297c; us-bis-export-0f7514b15e893f05152ab60895ba05e2f04eab02</t>
+          <t>us-bis-export-4dde4d81c422e0f99b9683ca4eb18c2392155e66; us-bis-export-f59ed2b7aa0178d73365395b38ded03461840d95; us-bis-export-43bd1392fc4f3113c614c4c2b359c7adb2e31d79; us-bis-export-bb0c4774e8ff1b1b178c383784b9f07610e38caf; us-bis-export-f48912305c4dbcc6bb8632385fc391070974773d; us-bis-export-41786fd0bd0a1322671f5091163b8bf2b12d149f; us-bis-export-995e9097a29d10642017db31ba22f09e344e297c; us-bis-export-02a71f0a0b4df2ec61183537fd02e6a84266b4a4; us-bis-export-535f1b58120e7716fa25ed80b1456b67c4156473; us-bis-export-9642b172a01249feb8ddeda82ac3d0d8b7b2bb90; us-bis-export-0f7514b15e893f05152ab60895ba05e2f04eab02; us-bis-export-9e57b0d8a1e9d2f89cc79b48ca81dc9ca509521d; us-bis-export-257a072ab7741aac127bbc27219b9e586a81fafd; us-bis-export-36fad77b3c3b0ed0ab420e0c78ba583f2c97eaec; us-bis-export-03a3131d777c0b0575f941d28b30cfac7a0bfe61; us-bis-export-634ad637ca4a0ae524073c800a55e83a6ca5b091; us-bis-export-ce7306e097264749e060f167284409070209a2c1</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
@@ -6090,7 +6098,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>cy-a23858f976cf121dbb0014dfb385cf0cdda413ac; cy-afeba2ac035744cffb623f27a1152f76b0d0ebb7; cy-f3b61a663b6de3cdc27b53e99e9c15b21d12961a; cy-29970d3344c0d0b2d67019015b8475dce8c38478; cy-8dd3eb80d265f75dad9a9a3d1359b4ff7801951f; cy-4d7b8e3ab7f31d5fd7e8623938d54286dd429556; NK-VRJum2fRYwvTJRm9xRNg84; cy-d3ee69c8b3ea70a47c58ba36b4bd3c98f4ae6cbb; cy-8389a85db6b70ffb8cb29d498a4d1e898ed069f5; cy-ee56eb8c443a7615cb2b80aa785d7ede2b599cfa; cy-ce05129da07e72c76a8d06820102b17ba60f9341; cy-d802e23b9fcbaacf8705ddde7a23cf0c447cf866; cy-223088d9245ddd2288b4990b254418c8ea8f1fce; cy-5b0538dfca5c3dfde24d94b4603942e73518c070; cy-4b132c7603b97c49a8b5b15b0da3106a1ea8d625; cy-79e79a017d1016b1e668e727688b1c9bfbe95854</t>
+          <t>cy-223088d9245ddd2288b4990b254418c8ea8f1fce; cy-d802e23b9fcbaacf8705ddde7a23cf0c447cf866; cy-4b132c7603b97c49a8b5b15b0da3106a1ea8d625; cy-afeba2ac035744cffb623f27a1152f76b0d0ebb7; cy-ce05129da07e72c76a8d06820102b17ba60f9341; cy-d3ee69c8b3ea70a47c58ba36b4bd3c98f4ae6cbb; cy-29970d3344c0d0b2d67019015b8475dce8c38478; cy-f3b61a663b6de3cdc27b53e99e9c15b21d12961a; NK-VRJum2fRYwvTJRm9xRNg84; cy-79e79a017d1016b1e668e727688b1c9bfbe95854; cy-8389a85db6b70ffb8cb29d498a4d1e898ed069f5; cy-ee56eb8c443a7615cb2b80aa785d7ede2b599cfa; cy-4d7b8e3ab7f31d5fd7e8623938d54286dd429556; cy-8dd3eb80d265f75dad9a9a3d1359b4ff7801951f; cy-a23858f976cf121dbb0014dfb385cf0cdda413ac; cy-5b0538dfca5c3dfde24d94b4603942e73518c070</t>
         </is>
       </c>
       <c r="H145" t="inlineStr"/>
@@ -6129,7 +6137,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>pk-cnic-3840359820147; pk-cnic-3120570621759; pk-cnic-3240271987885; pk-cnic-3240413956031; pk-cnic-3320267483611; pk-cnic-3840320506127; pk-cnic-3310280324005; pk-cnic-5340256608773; pk-cnic-5630110723091; pk-cnic-5550103456497; Q85739406; pk-cnic-3320371645081; pk-cnic-3540116384153; pk-cnic-4230138896977; pk-cnic-3840177568133; Q109767291</t>
+          <t>pk-cnic-3540116384153; pk-cnic-3320371645081; pk-cnic-3240413956031; pk-cnic-3840177568133; Q85739406; pk-cnic-3320267483611; pk-cnic-3120570621759; pk-cnic-3840359820147; pk-cnic-5550103456497; pk-cnic-3310280324005; pk-cnic-5630110723091; Q109767291; pk-cnic-3840320506127; pk-cnic-4230138896977; pk-cnic-3240271987885; pk-cnic-5340256608773</t>
         </is>
       </c>
       <c r="H146" t="inlineStr"/>
@@ -6168,7 +6176,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>isin-RU000A10BNK8; isin-RU000A10C5Z7; isin-RU000A109B82; isin-RU000A10CRB6; isin-RU000A109890; isin-RU000A10B4X6; isin-RU000A10BT00; isin-RU000A10D3S6; isin-RU000A10C3M0; isin-RU000A10BVF1; isin-RU000A10A026; isin-RU000A10B3Y6; isin-RU000A10BBE6; isin-RU000A10BY52; isin-RU000A108ZU2; isin-RU000A10ASD4</t>
+          <t>isin-RU000A10A026; isin-RU000A10C5Z7; isin-RU000A109890; isin-RU000A10BNK8; isin-RU000A10BVF1; isin-RU000A10D3S6; isin-RU000A108ZU2; isin-RU000A10ASD4; isin-RU000A109B82; isin-RU000A10B3Y6; isin-RU000A10BBE6; isin-RU000A10CRB6; isin-RU000A10C3M0; isin-RU000A10BT00; isin-RU000A10BY52; isin-RU000A10B4X6</t>
         </is>
       </c>
       <c r="H147" t="inlineStr"/>
@@ -6207,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>ru-inn-9718180638; ru-inn-5047263660; ru-inn-5643022352; ru-inn-3311024680; ru-inn-3849037461; ru-inn-7705555702; ru-inn-5044047196; ru-inn-5260478292; ru-inn-9108122988; ru-inn-7448136590; ru-inn-7714966755; ru-inn-7716873898; ru-inn-9701171900; ru-inn-9731150128; ru-inn-4307020290; ru-inn-1800001982</t>
+          <t>ru-inn-3849037461; ru-inn-5047263660; ru-inn-3311024680; ru-inn-9701171900; ru-inn-7714966755; ru-inn-9731150128; ru-inn-5260478292; ru-inn-9718180638; ru-inn-7448136590; ru-inn-7716873898; ru-inn-7705555702; ru-inn-4307020290; ru-inn-5044047196; ru-inn-5643022352; ru-inn-9108122988; ru-inn-1800001982</t>
         </is>
       </c>
       <c r="H148" t="inlineStr"/>
@@ -6246,7 +6254,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>ru-inn-7841098406; ru-inn-2221222189; ru-inn-9731069244; ru-inn-4205327082; ru-inn-9715422085; ru-inn-5048018929; ru-inn-7805250052; ru-inn-5038111005; ru-inn-9714059359; ru-inn-4826127992; ru-inn-9729006751; ru-inn-4252000920; ru-inn-7725371453; ru-inn-7707430353; ru-inn-7713495327; ru-inn-5257125360</t>
+          <t>ru-inn-7725371453; ru-inn-5038111005; ru-inn-7841098406; ru-inn-9731069244; ru-inn-4252000920; ru-inn-2221222189; ru-inn-9714059359; ru-inn-4826127992; ru-inn-7707430353; ru-inn-9729006751; ru-inn-9715422085; ru-inn-4205327082; ru-inn-7805250052; ru-inn-5257125360; ru-inn-5048018929; ru-inn-7713495327</t>
         </is>
       </c>
       <c r="H149" t="inlineStr"/>
@@ -6285,7 +6293,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>ua-edr-5d094c3ddabaa0437cd1b69ecc5b488bf77d38f0; ua-edr-e9b1aa90d0ad3e259df32472efe032ad4841b391; ua-edr-5af61c1a7efbccf8ae56504a447d8d84f1fd4dea; ua-edr-5e5ca2182dd3bcf0956a2d6c4e86a9f797dd4ba0; ua-edr-a5acd52925972aadcda603231fafc1282f41a1fe; ua-edr-4e1a6057dbb02f9a0b2cc6ceb3871b87ef2fd53c; ua-edr-d86dbb88879c1599e78c6f5e787730bed6e32aa4; ua-edr-9472168f49fb20e1f1753e691baa240e224265c9; ua-edr-ca1159568f1d4eec560aed6a9a5bae8d46dcba28; ua-edr-3ea3da70f834441deb8f77c450f28457bc1e8b1a; ua-edr-22154614206aa9662c46f509ce04b1103dd9a297; ua-edr-c6d42d5b4e212aafc7207f7557f33b4654e4917c; ua-edr-cede6ceb18599f5f73914e1f4ed83e42dfca5342; ua-edr-4242168f1602d66b7396365d8a2962f379c89686; ua-edr-5483750ea8a6040702cf8e6ee08911e13984cc18; ua-edr-82b0c874b4a03e4409d92323cdf16f13a4cb3cd4</t>
+          <t>ua-edr-82b0c874b4a03e4409d92323cdf16f13a4cb3cd4; ua-edr-ca1159568f1d4eec560aed6a9a5bae8d46dcba28; ua-edr-4e1a6057dbb02f9a0b2cc6ceb3871b87ef2fd53c; ua-edr-5d094c3ddabaa0437cd1b69ecc5b488bf77d38f0; ua-edr-5e5ca2182dd3bcf0956a2d6c4e86a9f797dd4ba0; ua-edr-e9b1aa90d0ad3e259df32472efe032ad4841b391; ua-edr-3ea3da70f834441deb8f77c450f28457bc1e8b1a; ua-edr-c6d42d5b4e212aafc7207f7557f33b4654e4917c; ua-edr-a5acd52925972aadcda603231fafc1282f41a1fe; ua-edr-d86dbb88879c1599e78c6f5e787730bed6e32aa4; ua-edr-5483750ea8a6040702cf8e6ee08911e13984cc18; ua-edr-22154614206aa9662c46f509ce04b1103dd9a297; ua-edr-4242168f1602d66b7396365d8a2962f379c89686; ua-edr-9472168f49fb20e1f1753e691baa240e224265c9; ua-edr-cede6ceb18599f5f73914e1f4ed83e42dfca5342; ua-edr-5af61c1a7efbccf8ae56504a447d8d84f1fd4dea</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
@@ -6324,7 +6332,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>cy-8a07910d7dd5f25ee391fe6e2640dd67454b6d2e; cy-2a20390a8c6760c606be6c7f8dabf1785bab8c51; cy-2e3e9e6cbc6b8a74eaa0d009cf4f99e27ef9fd8b; cy-90e2bb1252c2a89cdd2457ec8bf867907305005a; cy-d9a18fb5f8d757145ea4131c7a5446fbfe9e0e6b; cy-5d37aafc2f4a74217ce0f096b9e3ee6442ee3754; cy-b0ec6aadac28597e7bcc503cd1b9a1115cedf151; cy-19a1e020d6e925c3c8c5e44d9636d3d84629f7ec; cy-65dd5c869dc51903bfd595c75216fb000a2f0f00; cy-0d1a41bbad9a884592094a643c65691b5c50b6a5; cy-bfbe84015d82dc0477b23fe768a0e10ec220bffb; cy-f149aa3addc53ce34e9108c136605044a1fc898e; cy-e87a101b317b996481ffb57f03fe3597bfc80765; cy-00a9ff29cf59b91407a36a8fcb3274cae24a2312; cy-c96782983263f75ffc723af2968a68b4b0e0bd45</t>
+          <t>cy-b0ec6aadac28597e7bcc503cd1b9a1115cedf151; cy-2e3e9e6cbc6b8a74eaa0d009cf4f99e27ef9fd8b; cy-8a07910d7dd5f25ee391fe6e2640dd67454b6d2e; cy-00a9ff29cf59b91407a36a8fcb3274cae24a2312; cy-5d37aafc2f4a74217ce0f096b9e3ee6442ee3754; cy-19a1e020d6e925c3c8c5e44d9636d3d84629f7ec; cy-c96782983263f75ffc723af2968a68b4b0e0bd45; cy-65dd5c869dc51903bfd595c75216fb000a2f0f00; cy-bfbe84015d82dc0477b23fe768a0e10ec220bffb; cy-d9a18fb5f8d757145ea4131c7a5446fbfe9e0e6b; cy-0d1a41bbad9a884592094a643c65691b5c50b6a5; cy-e87a101b317b996481ffb57f03fe3597bfc80765; cy-2a20390a8c6760c606be6c7f8dabf1785bab8c51; cy-90e2bb1252c2a89cdd2457ec8bf867907305005a; cy-f149aa3addc53ce34e9108c136605044a1fc898e</t>
         </is>
       </c>
       <c r="H151" t="inlineStr"/>
@@ -7638,17 +7646,17 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>SECO UKRAINE vessel Russia</t>
+          <t>EU MARE vessel Russia</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>SECO UKRAINE ship Russia</t>
+          <t>EU MARE ship Russia</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>SECO UKRAINE vessel RU</t>
+          <t>EU MARE vessel RU</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -7658,7 +7666,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>programId=SECO-UKRAINE | schema=Vessel | country=ru</t>
+          <t>programId=EU-MARE | schema=Vessel | country=ru</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -7681,17 +7689,17 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>EU MARE vessel Russia</t>
+          <t>SECO UKRAINE vessel Russia</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>EU MARE ship Russia</t>
+          <t>SECO UKRAINE ship Russia</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>EU MARE vessel RU</t>
+          <t>SECO UKRAINE vessel RU</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -7701,7 +7709,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>programId=EU-MARE | schema=Vessel | country=ru</t>
+          <t>programId=SECO-UKRAINE | schema=Vessel | country=ru</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -7724,17 +7732,17 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>US DDTC SD person US</t>
+          <t>US AECA DEBARRED person US</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>US DDTC SD individual US</t>
+          <t>US AECA DEBARRED individual US</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>US DDTC SD person US</t>
+          <t>US AECA DEBARRED person US</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -7744,7 +7752,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>programId=US-DDTC-SD | schema=Person | country=us</t>
+          <t>programId=US-AECA-DEBARRED | schema=Person | country=us</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -7767,17 +7775,17 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>US AECA DEBARRED person US</t>
+          <t>US DDTC SD person US</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>US AECA DEBARRED individual US</t>
+          <t>US DDTC SD individual US</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>US AECA DEBARRED person US</t>
+          <t>US DDTC SD person US</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -7787,7 +7795,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>programId=US-AECA-DEBARRED | schema=Person | country=us</t>
+          <t>programId=US-DDTC-SD | schema=Person | country=us</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">

</xml_diff>